<commit_message>
Better syntax for fab copper layers and testpoints
</commit_message>
<xml_diff>
--- a/amulet_controller/Manufacturing/Assembly/amulet_controller-bom.xlsx
+++ b/amulet_controller/Manufacturing/Assembly/amulet_controller-bom.xlsx
@@ -725,16 +725,16 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.13      $0.13
-    10   $0.02      $0.21
-    50   $0.01      $0.74
-   100   $0.01      $1.31
-   500   $0.01      $4.98
-  1000   $0.01      $8.91
-  2500   $0.01     $19.50
-  5000   $0.01     $35.45
- 10000   $0.01     $65.00
- 50000   $0.01    $273.00</t>
+     1   $0.12      $0.12
+    10   $0.02      $0.20
+    50   $0.01      $0.73
+   100   $0.01      $1.29
+   500   $0.01      $4.91
+  1000   $0.01      $8.80
+  2500   $0.01     $19.25
+  5000   $0.01     $35.00
+ 10000   $0.01     $64.20
+ 50000   $0.01    $269.50</t>
         </r>
       </text>
     </comment>
@@ -854,7 +854,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>11534 In Stock</t>
+          <t>11515 In Stock</t>
         </r>
       </text>
     </comment>
@@ -952,7 +952,8 @@
    100   $0.08      $7.83
    500   $0.06     $29.75
   1000   $0.05     $53.60
-  2000   $0.05     $97.60</t>
+  2000   $0.05     $97.60
+  4000   $0.05    $194.40</t>
         </r>
       </text>
     </comment>
@@ -982,7 +983,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>100854 In Stock</t>
+          <t>48696 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1075,7 +1076,7 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
- 50000   $0.01    $340.00</t>
+ 50000   $0.01    $339.50</t>
         </r>
       </text>
     </comment>
@@ -1105,7 +1106,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>92659 In Stock</t>
+          <t>91233 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1194,7 +1195,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>2218056 In Stock</t>
+          <t>2175990 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1288,14 +1289,14 @@
 ================
      1   $0.09      $0.09
     10   $0.02      $0.19
-    50   $0.01      $0.67
-   100   $0.01      $1.16
-  1000   $0.01      $7.72
-  2500   $0.01     $16.77
-  5000   $0.01     $30.45
- 10000   $0.01     $55.80
-500000   $0.00  $1,960.00
-1000000   $0.00  $3,760.00</t>
+    50   $0.01      $0.66
+   100   $0.01      $1.15
+  1000   $0.01      $7.62
+  2500   $0.01     $16.55
+  5000   $0.01     $30.10
+ 10000   $0.01     $55.10
+500000   $0.00  $1,930.00
+1000000   $0.00  $3,710.00</t>
         </r>
       </text>
     </comment>
@@ -1424,7 +1425,7 @@
   1000   $0.04     $40.20
   2000   $0.04     $73.60
   4000   $0.03    $136.00
-  8000   $0.03    $250.40
+  8000   $0.03    $251.20
  12000   $0.03    $361.20</t>
         </r>
       </text>
@@ -1455,7 +1456,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>142639 In Stock</t>
+          <t>141969 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1544,7 +1545,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>60986 In Stock</t>
+          <t>This part is listed but is not stocked.</t>
         </r>
       </text>
     </comment>
@@ -1650,7 +1651,7 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
- 40000   $0.01    $408.00</t>
+ 40000   $0.01    $404.00</t>
         </r>
       </text>
     </comment>
@@ -1680,7 +1681,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>167930 In Stock</t>
+          <t>167430 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1769,7 +1770,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>18200 In Stock</t>
+          <t>17460 In Stock</t>
         </r>
       </text>
     </comment>
@@ -1865,15 +1866,15 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $0.09      $0.09
-    10   $0.04      $0.35
-    50   $0.03      $1.33
-   100   $0.02      $2.39
-  1000   $0.02     $16.70
-  2500   $0.01     $36.25
- 10000   $0.01    $118.00
- 50000   $0.01    $470.00
- 70000   $0.01    $623.00
-100000   $0.01    $850.00</t>
+    10   $0.03      $0.35
+    50   $0.03      $1.31
+   100   $0.02      $2.36
+  1000   $0.02     $16.40
+  2500   $0.01     $35.75
+ 10000   $0.01    $117.00
+ 50000   $0.01    $460.00
+ 70000   $0.01    $616.00
+100000   $0.01    $840.00</t>
         </r>
       </text>
     </comment>
@@ -2087,16 +2088,16 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.25      $0.25
-    10   $0.10      $1.05
-    50   $0.08      $4.12
-   100   $0.08      $7.52
-  1000   $0.06     $56.90
-  2500   $0.05    $129.00
- 10000   $0.05    $451.00
- 20000   $0.04    $850.00
- 50000   $0.04  $1,975.00
-100000   $0.04  $3,760.00</t>
+     1   $0.24      $0.24
+    10   $0.10      $1.03
+    50   $0.08      $4.08
+   100   $0.07      $7.42
+  1000   $0.06     $56.20
+  2500   $0.05    $127.50
+ 10000   $0.04    $446.00
+ 20000   $0.04    $840.00
+ 50000   $0.04  $1,950.00
+100000   $0.04  $3,710.00</t>
         </r>
       </text>
     </comment>
@@ -2126,7 +2127,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>18868 In Stock</t>
+          <t>18768 In Stock</t>
         </r>
       </text>
     </comment>
@@ -2148,7 +2149,7 @@
    500 CHF0.29  CHF145.50
   1000 CHF0.27  CHF265.00
   2000 CHF0.23  CHF452.00
- 10000 CHF0.20 CHF2,040.00</t>
+ 10000 CHF0.21 CHF2,070.00</t>
         </r>
       </text>
     </comment>
@@ -2217,15 +2218,15 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.88      $0.88
-     5   $0.49      $2.45
-    10   $0.45      $4.54
-    50   $0.38     $18.95
-   100   $0.35     $34.70
-   250   $0.31     $76.50
-   500   $0.28    $137.50
-  1000   $0.24    $244.00
-  2000   $0.21    $426.00</t>
+     1   $0.87      $0.87
+     5   $0.48      $2.42
+    10   $0.45      $4.48
+    50   $0.37     $18.70
+   100   $0.34     $34.30
+   250   $0.30     $75.50
+   500   $0.27    $136.00
+  1000   $0.24    $241.00
+  2000   $0.21    $420.00</t>
         </r>
       </text>
     </comment>
@@ -2255,7 +2256,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>18868 In Stock</t>
+          <t>18768 In Stock</t>
         </r>
       </text>
     </comment>
@@ -2277,7 +2278,7 @@
    500 CHF0.29  CHF145.50
   1000 CHF0.27  CHF265.00
   2000 CHF0.23  CHF452.00
- 10000 CHF0.20 CHF2,040.00</t>
+ 10000 CHF0.21 CHF2,070.00</t>
         </r>
       </text>
     </comment>
@@ -2346,15 +2347,15 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.88      $0.88
-     5   $0.49      $2.45
-    10   $0.45      $4.54
-    50   $0.38     $18.95
-   100   $0.35     $34.70
-   250   $0.31     $76.50
-   500   $0.28    $137.50
-  1000   $0.24    $244.00
-  2000   $0.21    $426.00</t>
+     1   $0.87      $0.87
+     5   $0.48      $2.42
+    10   $0.45      $4.48
+    50   $0.37     $18.70
+   100   $0.34     $34.30
+   250   $0.30     $75.50
+   500   $0.27    $136.00
+  1000   $0.24    $241.00
+  2000   $0.21    $420.00</t>
         </r>
       </text>
     </comment>
@@ -2489,7 +2490,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>140098 In Stock</t>
+          <t>135928 In Stock</t>
         </r>
       </text>
     </comment>
@@ -2595,14 +2596,14 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $0.35      $0.35
-    10   $0.23      $2.34
-    50   $0.16      $7.90
-   100   $0.14     $13.50
-   500   $0.10     $49.00
-  1000   $0.09     $88.00
-  3000   $0.08    $228.00
- 15000   $0.07    $990.00
- 75000   $0.06  $4,725.00</t>
+    10   $0.23      $2.31
+    50   $0.16      $7.80
+   100   $0.13     $13.30
+   500   $0.10     $48.00
+  1000   $0.09     $87.00
+  3000   $0.07    $225.00
+ 15000   $0.07    $975.00
+ 75000   $0.06  $4,650.00</t>
         </r>
       </text>
     </comment>
@@ -2632,7 +2633,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>2614 In Stock</t>
+          <t>2414 In Stock</t>
         </r>
       </text>
     </comment>
@@ -2734,8 +2735,8 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-  1000   $0.54    $542.00
-  7000   $0.52  $3,612.00</t>
+  1000   $0.54    $543.00
+  7000   $0.52  $3,605.00</t>
         </r>
       </text>
     </comment>
@@ -2765,7 +2766,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>41033 In Stock</t>
+          <t>21268 In Stock</t>
         </r>
       </text>
     </comment>
@@ -2781,13 +2782,12 @@
           <t>Qty/Price Breaks (CHF):
   Qty  -  UnitCHF  -  ExtCHF
 ================
-     1 CHF0.36    CHF0.36
-    10 CHF0.15    CHF1.53
-   100 CHF0.10   CHF10.40
-  1000 CHF0.10   CHF95.00
-  3000 CHF0.08  CHF228.00
-  9000 CHF0.07  CHF612.00
- 24000 CHF0.07 CHF1,560.00
+     1 CHF0.37    CHF0.37
+    10 CHF0.16    CHF1.58
+   100 CHF0.11   CHF10.80
+  1000 CHF0.10   CHF98.00
+  3000 CHF0.08  CHF243.00
+  9000 CHF0.08  CHF711.00
  45000 CHF0.06 CHF2,745.00
  99000 CHF0.06 CHF5,841.00</t>
         </r>
@@ -2871,16 +2871,16 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1   $0.33      $0.33
-     5   $0.23      $1.15
-    10   $0.19      $1.87
-    50   $0.12      $6.10
-   100   $0.10     $10.50
-  1000   $0.08     $79.00
-  3000   $0.07    $225.00
-  6000   $0.07    $438.00
-  9000   $0.07    $648.00
- 45000   $0.07  $3,150.00</t>
+     1   $0.32      $0.32
+     5   $0.23      $1.13
+    10   $0.18      $1.85
+    50   $0.12      $6.00
+   100   $0.10     $10.40
+  1000   $0.08     $78.00
+  3000   $0.07    $222.00
+  6000   $0.07    $432.00
+  9000   $0.07    $639.00
+ 45000   $0.07  $3,105.00</t>
         </r>
       </text>
     </comment>
@@ -3108,9 +3108,9 @@
     50   $0.14      $7.24
    100   $0.10      $9.55
   1000   $0.08     $84.80
-  2500   $0.07    $176.00
+  2500   $0.07    $176.25
   3000   $0.07    $200.70
-  6000   $0.06    $373.20
+  6000   $0.06    $373.80
   9000   $0.06    $517.50
  45000   $0.06  $2,529.00</t>
         </r>
@@ -3139,7 +3139,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>42722 In Stock</t>
+          <t>40692 In Stock</t>
         </r>
       </text>
     </comment>
@@ -3226,9 +3226,9 @@
      1   $1.84      $1.84
     10   $0.84      $8.41
    100   $0.64     $64.10
-   500   $0.55    $275.50
-  1000   $0.52    $522.00
-  1500   $0.51    $759.00
+   500   $0.55    $276.00
+  1000   $0.52    $523.00
+  1500   $0.51    $760.50
   3000   $0.48  $1,452.00
   6000   $0.46  $2,778.00</t>
         </r>
@@ -3258,7 +3258,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>13265 In Stock</t>
+          <t>13255 In Stock</t>
         </r>
       </text>
     </comment>
@@ -3341,7 +3341,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>11191 In Stock</t>
+          <t>11091 In Stock</t>
         </r>
       </text>
     </comment>
@@ -3689,7 +3689,7 @@
      1   $0.38      $0.38
     10   $0.28      $2.84
    100   $0.19     $19.30
-   500   $0.14     $71.00
+   500   $0.14     $71.50
    750   $0.13     $98.25
   1500   $0.11    $168.00
   2250   $0.10    $231.75</t>
@@ -3818,7 +3818,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>20355 In Stock</t>
+          <t>20255 In Stock</t>
         </r>
       </text>
     </comment>
@@ -4027,7 +4027,7 @@
   Qty  -  Unit$  -  Ext$
 ================
      5   $0.30      $1.48
-    20   $0.25      $5.06
+    20   $0.25      $5.08
    100   $0.21     $21.20
    500   $0.17     $85.00</t>
         </r>
@@ -4235,10 +4235,10 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $0.82      $0.82
-    10   $0.71      $7.15
+    10   $0.72      $7.16
    100   $0.62     $61.60
    500   $0.51    $256.50
-  1000   $0.41    $409.00</t>
+  1000   $0.41    $410.00</t>
         </r>
       </text>
     </comment>
@@ -4400,9 +4400,9 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $0.93      $0.93
-    10   $0.81      $8.10
-   100   $0.70     $69.70
-   500   $0.58    $291.00
+    10   $0.81      $8.11
+   100   $0.70     $69.80
+   500   $0.58    $291.50
   1000   $0.46    $464.00</t>
         </r>
       </text>
@@ -4541,7 +4541,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>38725 In Stock</t>
+          <t>38720 In Stock</t>
         </r>
       </text>
     </comment>
@@ -4708,7 +4708,7 @@
 ================
      1   $0.53      $0.53
     10   $0.40      $4.00
-    25   $0.31      $7.78
+    25   $0.31      $7.80
    100   $0.20     $20.10
    500   $0.14     $67.50
   1000   $0.12    $121.00
@@ -4852,7 +4852,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>8933 In Stock</t>
+          <t>8867 In Stock</t>
         </r>
       </text>
     </comment>
@@ -4944,7 +4944,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>1005696 In Stock</t>
+          <t>985110 In Stock</t>
         </r>
       </text>
     </comment>
@@ -5074,7 +5074,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>461985 In Stock</t>
+          <t>460545 In Stock</t>
         </r>
       </text>
     </comment>
@@ -5201,7 +5201,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>7045 In Stock</t>
+          <t>6935 In Stock</t>
         </r>
       </text>
     </comment>
@@ -5293,7 +5293,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>13400 In Stock</t>
+          <t>13350 In Stock</t>
         </r>
       </text>
     </comment>
@@ -5518,7 +5518,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>206603 In Stock</t>
+          <t>206254 In Stock</t>
         </r>
       </text>
     </comment>
@@ -5937,7 +5937,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>868580 In Stock</t>
+          <t>867700 In Stock</t>
         </r>
       </text>
     </comment>
@@ -6033,7 +6033,7 @@
     50   $0.02      $0.76
    100   $0.01      $1.10
   1000   $0.01      $5.24
-  2500   $0.00     $11.38
+  2500   $0.00     $11.40
  10000   $0.00     $40.90
 500000   $0.00  $1,920.00
 1000000   $0.00  $3,810.00</t>
@@ -6247,7 +6247,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>146709 In Stock</t>
+          <t>145019 In Stock</t>
         </r>
       </text>
     </comment>
@@ -6344,9 +6344,9 @@
    100   $0.02      $1.60
    500   $0.01      $7.33
   1000   $0.01     $12.98
-  2500   $0.01     $25.05
+  2500   $0.01     $25.08
   3000   $0.01     $29.13
-  5000   $0.01     $43.25
+  5000   $0.01     $43.30
  10000   $0.00     $38.00</t>
         </r>
       </text>
@@ -6378,7 +6378,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>191994 In Stock</t>
+          <t>191844 In Stock</t>
         </r>
       </text>
     </comment>
@@ -6618,14 +6618,14 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $0.13      $0.13
-    10   $0.10      $0.98
-    50   $0.08      $4.04
-   100   $0.07      $7.45
-   500   $0.06     $31.15
-  1000   $0.06     $58.10
-  2500   $0.05    $132.75
- 10000   $0.05    $471.00
-250000   $0.04  $9,425.00</t>
+    10   $0.10      $0.96
+    50   $0.08      $3.99
+   100   $0.07      $7.35
+   500   $0.06     $30.75
+  1000   $0.06     $57.30
+  2500   $0.05    $131.00
+ 10000   $0.05    $465.00
+250000   $0.04  $9,300.00</t>
         </r>
       </text>
     </comment>
@@ -6654,7 +6654,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>6462 In Stock</t>
+          <t>6446 In Stock</t>
         </r>
       </text>
     </comment>
@@ -6814,7 +6814,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>3465 In Stock</t>
+          <t>3365 In Stock</t>
         </r>
       </text>
     </comment>
@@ -6919,8 +6919,8 @@
      1   $0.93      $0.93
      5   $0.62      $3.08
     25   $0.58     $14.50
-   100   $0.55     $54.70
-   500   $0.51    $253.00
+   100   $0.55     $54.80
+   500   $0.51    $253.50
   3000   $0.46  $1,386.00
   6000   $0.43  $2,580.00
  12000   $0.40  $4,800.00</t>
@@ -7426,7 +7426,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>4812 In Stock</t>
+          <t>4752 In Stock</t>
         </r>
       </text>
     </comment>
@@ -7637,14 +7637,14 @@
           <t>Qty/Price Breaks (USD):
   Qty  -  Unit$  -  Ext$
 ================
-     1  $10.76     $10.76
-     3  $10.23     $30.69
+     1  $10.77     $10.77
+     3  $10.24     $30.72
     10   $9.73     $97.30
     25   $9.17    $229.25
     50   $8.61    $430.50
    100   $8.05    $805.00
    250   $7.27  $1,817.50
-   500   $6.99  $3,495.00
+   500   $7.00  $3,500.00
   1000   $6.71  $6,710.00</t>
         </r>
       </text>
@@ -7757,7 +7757,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>6702 In Stock</t>
+          <t>6682 In Stock</t>
         </r>
       </text>
     </comment>
@@ -7847,15 +7847,15 @@
   Qty  -  Unit$  -  Ext$
 ================
      1   $1.23      $1.23
-    10   $1.08     $10.84
-    50   $0.91     $45.45
-   100   $0.83     $83.20
-   250   $0.74    $184.50
-   500   $0.67    $337.00
+    10   $1.08     $10.85
+    50   $0.91     $45.50
+   100   $0.83     $83.30
+   250   $0.74    $184.75
+   500   $0.68    $337.50
   1000   $0.61    $615.00
-  2500   $0.55  $1,362.50
+  2500   $0.55  $1,365.00
   3000   $0.53  $1,599.00
-  9000   $0.52  $4,707.00</t>
+  9000   $0.52  $4,716.00</t>
         </r>
       </text>
     </comment>
@@ -7944,7 +7944,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3921" uniqueCount="1496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3922" uniqueCount="1496">
   <si>
     <t>Row</t>
   </si>
@@ -9626,7 +9626,7 @@
     <t>Variant:</t>
   </si>
   <si>
-    <t>RELEASED</t>
+    <t>default</t>
   </si>
   <si>
     <t>Revision:</t>
@@ -9728,6 +9728,9 @@
     <t>81-GRM155Z71A105KE1J</t>
   </si>
   <si>
+    <t>NonStk</t>
+  </si>
+  <si>
     <t>963-TMK107AB7105KAHT</t>
   </si>
   <si>
@@ -9743,9 +9746,6 @@
     <t>581-04023D475MAT2A</t>
   </si>
   <si>
-    <t>NonStk</t>
-  </si>
-  <si>
     <t>81-GRM21BZ71E106KE5L</t>
   </si>
   <si>
@@ -9944,7 +9944,7 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2024-11-20 18:33:31</t>
+    <t>2024-11-21 22:58:15</t>
   </si>
   <si>
     <t>KiCost® v1.1.18 + KiBot v1.8.3</t>
@@ -16596,7 +16596,7 @@
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
-        <v>144.735</v>
+        <v>144.5116</v>
       </c>
     </row>
     <row r="4" spans="1:26">
@@ -16611,11 +16611,11 @@
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H80)</f>
-        <v>144.735</v>
+        <v>144.5116</v>
       </c>
       <c r="M4" s="16">
         <f>SUM(M10:M80)</f>
-        <v>142.3756</v>
+        <v>142.6412</v>
       </c>
       <c r="N4" s="17" t="str">
         <f>(COUNTA(M10:M80)&amp;" of "&amp;ROWS(M10:M80)&amp;" parts found")</f>
@@ -16631,7 +16631,7 @@
       </c>
       <c r="Y4" s="16">
         <f>SUM(Y10:Y80)</f>
-        <v>58.3769</v>
+        <v>58.0649</v>
       </c>
       <c r="Z4" s="17" t="str">
         <f>(COUNTA(Y10:Y80)&amp;" of "&amp;ROWS(Y10:Y80)&amp;" parts found")</f>
@@ -16804,14 +16804,14 @@
       <c r="J10" s="23"/>
       <c r="K10" s="24">
         <f>IFERROR(IF(OR(J10&gt;=L10,F10&gt;=L10),USD_CHF*LOOKUP(IF(J10="",F10,J10),{0,1,10,100,1000,10000,50000},{0.0,0.091,0.024,0.015,0.009,0.007,0.006}),"MOQ="&amp;L10),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L10" s="23">
         <v>1</v>
       </c>
       <c r="M10" s="25">
         <f>IFERROR(IF(J10="",F10,J10)*K10,"")</f>
-        <v>0.3087</v>
+        <v>0.3092</v>
       </c>
       <c r="N10" s="23" t="s">
         <v>583</v>
@@ -16869,14 +16869,14 @@
       <c r="J11" s="23"/>
       <c r="K11" s="24">
         <f>IFERROR(IF(OR(J11&gt;=L11,F11&gt;=L11),USD_CHF*LOOKUP(IF(J11="",F11,J11),{0,1,10,100,1000,2500,10000,20000},{0.0,0.091,0.024,0.017,0.014,0.01,0.008,0.007}),"MOQ="&amp;L11),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L11" s="23">
         <v>1</v>
       </c>
       <c r="M11" s="25">
         <f>IFERROR(IF(J11="",F11,J11)*K11,"")</f>
-        <v>0.6173</v>
+        <v>0.6184</v>
       </c>
       <c r="N11" s="23" t="s">
         <v>584</v>
@@ -16934,14 +16934,14 @@
       <c r="J12" s="23"/>
       <c r="K12" s="24">
         <f>IFERROR(IF(OR(J12&gt;=L12,F12&gt;=L12),USD_CHF*LOOKUP(IF(J12="",F12,J12),{0,1,10,100,2500,10000,50000},{0.0,0.091,0.015,0.008,0.006,0.005,0.004}),"MOQ="&amp;L12),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L12" s="23">
         <v>1</v>
       </c>
       <c r="M12" s="25">
         <f>IFERROR(IF(J12="",F12,J12)*K12,"")</f>
-        <v>0.1029</v>
+        <v>0.1031</v>
       </c>
       <c r="N12" s="23" t="s">
         <v>585</v>
@@ -16969,15 +16969,15 @@
       </c>
       <c r="V12" s="23"/>
       <c r="W12" s="24">
-        <f>IFERROR(IF(OR(V12&gt;=X12,F12&gt;=X12),LOOKUP(IF(V12="",F12,V12),{0,1,10,50,100,500,1000,2500,5000,10000,50000},{0.0,0.1252,0.02068,0.01489,0.01307,0.00995,0.00891,0.0078,0.00709,0.0065,0.00546}),"MOQ="&amp;X12),"")</f>
-        <v>0.1252</v>
+        <f>IFERROR(IF(OR(V12&gt;=X12,F12&gt;=X12),LOOKUP(IF(V12="",F12,V12),{0,1,10,50,100,500,1000,2500,5000,10000,50000},{0.0,0.12358,0.02041,0.0147,0.0129,0.00982,0.0088,0.0077,0.007,0.00642,0.00539}),"MOQ="&amp;X12),"")</f>
+        <v>0.12358</v>
       </c>
       <c r="X12" s="23">
         <v>1</v>
       </c>
       <c r="Y12" s="25">
         <f>IFERROR(IF(V12="",F12,V12)*W12,"")</f>
-        <v>0.1252</v>
+        <v>0.1236</v>
       </c>
       <c r="Z12" s="23" t="s">
         <v>43</v>
@@ -17017,14 +17017,14 @@
       <c r="J13" s="23"/>
       <c r="K13" s="24">
         <f>IFERROR(IF(OR(J13&gt;=L13,F13&gt;=L13),USD_CHF*LOOKUP(IF(J13="",F13,J13),{0,1,10,100,1000,2500,10000,50000},{0.0,0.145,0.097,0.048,0.031,0.029,0.023,0.022}),"MOQ="&amp;L13),"")</f>
-        <v>0.1639359880111325</v>
+        <v>0.16422100279750376</v>
       </c>
       <c r="L13" s="23">
         <v>1</v>
       </c>
       <c r="M13" s="25">
         <f>IFERROR(IF(J13="",F13,J13)*K13,"")</f>
-        <v>0.1639</v>
+        <v>0.1642</v>
       </c>
       <c r="N13" s="23" t="s">
         <v>586</v>
@@ -17070,32 +17070,32 @@
       </c>
       <c r="G14" s="24">
         <f>IF(MIN(Q14,K14,W14)&lt;&gt;0,MIN(Q14,K14,W14),"")</f>
-        <v>0.2304</v>
+        <v>0.2305</v>
       </c>
       <c r="H14" s="25">
         <f>IF(AND(ISNUMBER(F14),ISNUMBER(G14)),F14*G14,"")</f>
-        <v>0.2304</v>
+        <v>0.2305</v>
       </c>
       <c r="I14" s="23">
-        <v>11534</v>
+        <v>11515</v>
       </c>
       <c r="J14" s="23"/>
       <c r="K14" s="24">
         <f>IFERROR(IF(OR(J14&gt;=L14,F14&gt;=L14),USD_CHF*LOOKUP(IF(J14="",F14,J14),{0,1,10,100,1000,4000,8000,24000,100000},{0.0,0.236,0.097,0.062,0.052,0.045,0.04,0.037,0.034}),"MOQ="&amp;L14),"")</f>
-        <v>0.2668199529008777</v>
+        <v>0.26728383903593717</v>
       </c>
       <c r="L14" s="23">
         <v>1</v>
       </c>
       <c r="M14" s="25">
         <f>IFERROR(IF(J14="",F14,J14)*K14,"")</f>
-        <v>0.2668</v>
+        <v>0.2673</v>
       </c>
       <c r="N14" s="23" t="s">
         <v>587</v>
       </c>
       <c r="O14" s="23">
-        <v>14356</v>
+        <v>14336</v>
       </c>
       <c r="P14" s="23"/>
       <c r="Q14" s="24">
@@ -17117,15 +17117,15 @@
       </c>
       <c r="V14" s="23"/>
       <c r="W14" s="24">
-        <f>IFERROR(IF(OR(V14&gt;=X14,F14&gt;=X14),LOOKUP(IF(V14="",F14,V14),{0,1,10,50,100,500,1000,2000},{0.0,0.2304,0.1248,0.0892,0.0783,0.0595,0.0536,0.0488}),"MOQ="&amp;X14),"")</f>
-        <v>0.2304</v>
+        <f>IFERROR(IF(OR(V14&gt;=X14,F14&gt;=X14),LOOKUP(IF(V14="",F14,V14),{0,1,10,50,100,500,1000,2000,4000},{0.0,0.2305,0.1249,0.0893,0.0783,0.0595,0.0536,0.0488,0.0486}),"MOQ="&amp;X14),"")</f>
+        <v>0.2305</v>
       </c>
       <c r="X14" s="23">
         <v>1</v>
       </c>
       <c r="Y14" s="25">
         <f>IFERROR(IF(V14="",F14,V14)*W14,"")</f>
-        <v>0.2304</v>
+        <v>0.2305</v>
       </c>
       <c r="Z14" s="23" t="s">
         <v>60</v>
@@ -17153,32 +17153,32 @@
       </c>
       <c r="G15" s="24">
         <f>IF(MIN(Q15,K15,W15)&lt;&gt;0,MIN(Q15,K15,W15),"")</f>
-        <v>0.02261186041532862</v>
+        <v>0.022651172799655696</v>
       </c>
       <c r="H15" s="25">
         <f>IF(AND(ISNUMBER(F15),ISNUMBER(G15)),F15*G15,"")</f>
-        <v>0.5879</v>
+        <v>0.5889</v>
       </c>
       <c r="I15" s="23">
-        <v>100854</v>
+        <v>48696</v>
       </c>
       <c r="J15" s="23"/>
       <c r="K15" s="24">
         <f>IFERROR(IF(OR(J15&gt;=L15,F15&gt;=L15),USD_CHF*LOOKUP(IF(J15="",F15,J15),{0,1,10,100,1000,2500,10000,50000},{0.0,0.091,0.02,0.013,0.01,0.008,0.007,0.007}),"MOQ="&amp;L15),"")</f>
-        <v>0.02261186041532862</v>
+        <v>0.022651172799655696</v>
       </c>
       <c r="L15" s="23">
         <v>1</v>
       </c>
       <c r="M15" s="25">
         <f>IFERROR(IF(J15="",F15,J15)*K15,"")</f>
-        <v>0.5879</v>
+        <v>0.5889</v>
       </c>
       <c r="N15" s="23" t="s">
         <v>588</v>
       </c>
       <c r="O15" s="23">
-        <v>2147752</v>
+        <v>2146412</v>
       </c>
       <c r="P15" s="23"/>
       <c r="Q15" s="24">
@@ -17200,7 +17200,7 @@
       </c>
       <c r="V15" s="23"/>
       <c r="W15" s="24">
-        <f>IFERROR(IF(OR(V15&gt;=X15,F15&gt;=X15),LOOKUP(IF(V15="",F15,V15),{0,1,50000},{0.0,0.0068,0.0068}),"MOQ="&amp;X15),"")</f>
+        <f>IFERROR(IF(OR(V15&gt;=X15,F15&gt;=X15),LOOKUP(IF(V15="",F15,V15),{0,1,50000},{0.0,0.00679,0.00679}),"MOQ="&amp;X15),"")</f>
         <v/>
       </c>
       <c r="X15" s="23">
@@ -17243,25 +17243,25 @@
         <v>0.3</v>
       </c>
       <c r="I16" s="23">
-        <v>92659</v>
+        <v>91233</v>
       </c>
       <c r="J16" s="23"/>
       <c r="K16" s="24">
         <f>IFERROR(IF(OR(J16&gt;=L16,F16&gt;=L16),USD_CHF*LOOKUP(IF(J16="",F16,J16),{0,1,10,100,1000,4000,8000,24000,48000},{0.0,0.137,0.053,0.033,0.025,0.02,0.017,0.016,0.015}),"MOQ="&amp;L16),"")</f>
-        <v>0.15489124384500105</v>
+        <v>0.15516053367764152</v>
       </c>
       <c r="L16" s="23">
         <v>1</v>
       </c>
       <c r="M16" s="25">
         <f>IFERROR(IF(J16="",F16,J16)*K16,"")</f>
-        <v>0.3098</v>
+        <v>0.3103</v>
       </c>
       <c r="N16" s="23" t="s">
         <v>589</v>
       </c>
       <c r="O16" s="23">
-        <v>387011</v>
+        <v>386999</v>
       </c>
       <c r="P16" s="23"/>
       <c r="Q16" s="24">
@@ -17301,32 +17301,32 @@
       </c>
       <c r="G17" s="24">
         <f>IF(MIN(Q17,K17,W17)&lt;&gt;0,MIN(Q17,K17,W17),"")</f>
-        <v>0.09203</v>
+        <v>0.09084</v>
       </c>
       <c r="H17" s="25">
         <f>IF(AND(ISNUMBER(F17),ISNUMBER(G17)),F17*G17,"")</f>
-        <v>0.092</v>
+        <v>0.0908</v>
       </c>
       <c r="I17" s="23">
-        <v>2218056</v>
+        <v>2175990</v>
       </c>
       <c r="J17" s="23"/>
       <c r="K17" s="24">
         <f>IFERROR(IF(OR(J17&gt;=L17,F17&gt;=L17),USD_CHF*LOOKUP(IF(J17="",F17,J17),{0,1,10,100,1000,2500,10000},{0.0,0.091,0.019,0.011,0.01,0.007,0.005}),"MOQ="&amp;L17),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L17" s="23">
         <v>1</v>
       </c>
       <c r="M17" s="25">
         <f>IFERROR(IF(J17="",F17,J17)*K17,"")</f>
-        <v>0.1029</v>
+        <v>0.1031</v>
       </c>
       <c r="N17" s="23" t="s">
         <v>590</v>
       </c>
       <c r="O17" s="23">
-        <v>812601</v>
+        <v>812501</v>
       </c>
       <c r="P17" s="23"/>
       <c r="Q17" s="24">
@@ -17348,15 +17348,15 @@
       </c>
       <c r="V17" s="23"/>
       <c r="W17" s="24">
-        <f>IFERROR(IF(OR(V17&gt;=X17,F17&gt;=X17),LOOKUP(IF(V17="",F17,V17),{0,1,10,50,100,1000,2500,5000,10000,500000,1000000},{0.0,0.09203,0.01912,0.01337,0.01164,0.00772,0.00671,0.00609,0.00558,0.00392,0.00376}),"MOQ="&amp;X17),"")</f>
-        <v>0.09203</v>
+        <f>IFERROR(IF(OR(V17&gt;=X17,F17&gt;=X17),LOOKUP(IF(V17="",F17,V17),{0,1,10,50,100,1000,2500,5000,10000,500000,1000000},{0.0,0.09084,0.01887,0.0132,0.01148,0.00762,0.00662,0.00602,0.00551,0.00386,0.00371}),"MOQ="&amp;X17),"")</f>
+        <v>0.09084</v>
       </c>
       <c r="X17" s="23">
         <v>1</v>
       </c>
       <c r="Y17" s="25">
         <f>IFERROR(IF(V17="",F17,V17)*W17,"")</f>
-        <v>0.092</v>
+        <v>0.0908</v>
       </c>
       <c r="Z17" s="23" t="s">
         <v>82</v>
@@ -17384,11 +17384,11 @@
       </c>
       <c r="G18" s="24">
         <f>IF(MIN(Q18,K18,W18)&lt;&gt;0,MIN(Q18,K18,W18),"")</f>
-        <v>0.2115</v>
+        <v>0.2116</v>
       </c>
       <c r="H18" s="25">
         <f>IF(AND(ISNUMBER(F18),ISNUMBER(G18)),F18*G18,"")</f>
-        <v>0.6345</v>
+        <v>0.6348</v>
       </c>
       <c r="I18" s="23">
         <v>23897</v>
@@ -17396,14 +17396,14 @@
       <c r="J18" s="23"/>
       <c r="K18" s="24">
         <f>IFERROR(IF(OR(J18&gt;=L18,F18&gt;=L18),USD_CHF*LOOKUP(IF(J18="",F18,J18),{0,1,10,100,1000,4000,8000,24000},{0.0,0.209,0.11,0.066,0.049,0.045,0.037,0.035}),"MOQ="&amp;L18),"")</f>
-        <v>0.23629394134018405</v>
+        <v>0.23670475575640199</v>
       </c>
       <c r="L18" s="23">
         <v>1</v>
       </c>
       <c r="M18" s="25">
         <f>IFERROR(IF(J18="",F18,J18)*K18,"")</f>
-        <v>0.7089</v>
+        <v>0.7101</v>
       </c>
       <c r="N18" s="23" t="s">
         <v>591</v>
@@ -17431,15 +17431,15 @@
       </c>
       <c r="V18" s="23"/>
       <c r="W18" s="24">
-        <f>IFERROR(IF(OR(V18&gt;=X18,F18&gt;=X18),LOOKUP(IF(V18="",F18,V18),{0,1,10,50,100,500,1000,2000,4000,8000,12000},{0.0,0.2115,0.08,0.0615,0.0554,0.0441,0.0402,0.0368,0.034,0.0313,0.0301}),"MOQ="&amp;X18),"")</f>
-        <v>0.2115</v>
+        <f>IFERROR(IF(OR(V18&gt;=X18,F18&gt;=X18),LOOKUP(IF(V18="",F18,V18),{0,1,10,50,100,500,1000,2000,4000,8000,12000},{0.0,0.2116,0.08,0.0615,0.0554,0.0441,0.0402,0.0368,0.034,0.0314,0.0301}),"MOQ="&amp;X18),"")</f>
+        <v>0.2116</v>
       </c>
       <c r="X18" s="23">
         <v>1</v>
       </c>
       <c r="Y18" s="25">
         <f>IFERROR(IF(V18="",F18,V18)*W18,"")</f>
-        <v>0.6345</v>
+        <v>0.6348</v>
       </c>
       <c r="Z18" s="23" t="s">
         <v>89</v>
@@ -17474,25 +17474,25 @@
         <v>0.5</v>
       </c>
       <c r="I19" s="23">
-        <v>142639</v>
+        <v>141969</v>
       </c>
       <c r="J19" s="23"/>
       <c r="K19" s="24">
         <f>IFERROR(IF(OR(J19&gt;=L19,F19&gt;=L19),USD_CHF*LOOKUP(IF(J19="",F19,J19),{0,1,10,100,1000,4000,8000,24000,100000},{0.0,0.227,0.093,0.059,0.046,0.044,0.035,0.033,0.032}),"MOQ="&amp;L19),"")</f>
-        <v>0.25664461571397984</v>
+        <v>0.2570908112760921</v>
       </c>
       <c r="L19" s="23">
         <v>1</v>
       </c>
       <c r="M19" s="25">
         <f>IFERROR(IF(J19="",F19,J19)*K19,"")</f>
-        <v>0.5133</v>
+        <v>0.5142</v>
       </c>
       <c r="N19" s="23" t="s">
         <v>592</v>
       </c>
       <c r="O19" s="23">
-        <v>92438</v>
+        <v>91083</v>
       </c>
       <c r="P19" s="23"/>
       <c r="Q19" s="24">
@@ -17538,26 +17538,26 @@
         <f>IF(AND(ISNUMBER(F20),ISNUMBER(G20)),F20*G20,"")</f>
         <v>0.5</v>
       </c>
-      <c r="I20" s="23">
-        <v>60986</v>
+      <c r="I20" s="26" t="s">
+        <v>594</v>
       </c>
       <c r="J20" s="23"/>
       <c r="K20" s="24">
         <f>IFERROR(IF(OR(J20&gt;=L20,F20&gt;=L20),USD_CHF*LOOKUP(IF(J20="",F20,J20),{0,1,10,100,1000,2500,10000,40000},{0.0,0.091,0.037,0.022,0.018,0.017,0.014,0.012}),"MOQ="&amp;L20),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L20" s="23">
         <v>1</v>
       </c>
       <c r="M20" s="25">
         <f>IFERROR(IF(J20="",F20,J20)*K20,"")</f>
-        <v>0.5144</v>
+        <v>0.5153</v>
       </c>
       <c r="N20" s="23" t="s">
         <v>593</v>
       </c>
       <c r="O20" s="23">
-        <v>270191</v>
+        <v>269676</v>
       </c>
       <c r="P20" s="23"/>
       <c r="Q20" s="24">
@@ -17575,11 +17575,11 @@
         <v>102</v>
       </c>
       <c r="U20" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V20" s="23"/>
       <c r="W20" s="24">
-        <f>IFERROR(IF(OR(V20&gt;=X20,F20&gt;=X20),LOOKUP(IF(V20="",F20,V20),{0,1,40000},{0.0,0.0102,0.0102}),"MOQ="&amp;X20),"")</f>
+        <f>IFERROR(IF(OR(V20&gt;=X20,F20&gt;=X20),LOOKUP(IF(V20="",F20,V20),{0,1,40000},{0.0,0.0101,0.0101}),"MOQ="&amp;X20),"")</f>
         <v/>
       </c>
       <c r="X20" s="23">
@@ -17622,22 +17622,22 @@
         <v>0.36</v>
       </c>
       <c r="I21" s="23">
-        <v>167930</v>
+        <v>167430</v>
       </c>
       <c r="J21" s="23"/>
       <c r="K21" s="24">
         <f>IFERROR(IF(OR(J21&gt;=L21,F21&gt;=L21),USD_CHF*LOOKUP(IF(J21="",F21,J21),{0,1,10,100,1000,4000,8000,24000,100000},{0.0,0.109,0.046,0.026,0.02,0.017,0.016,0.014,0.012}),"MOQ="&amp;L21),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="L21" s="23">
         <v>1</v>
       </c>
       <c r="M21" s="25">
         <f>IFERROR(IF(J21="",F21,J21)*K21,"")</f>
-        <v>0.3697</v>
+        <v>0.3703</v>
       </c>
       <c r="N21" s="23" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="O21" s="23">
         <v>618650</v>
@@ -17680,29 +17680,29 @@
       </c>
       <c r="G22" s="24">
         <f>IF(MIN(Q22,K22,W22)&lt;&gt;0,MIN(Q22,K22,W22),"")</f>
-        <v>0.092</v>
+        <v>0.0908</v>
       </c>
       <c r="H22" s="25">
         <f>IF(AND(ISNUMBER(F22),ISNUMBER(G22)),F22*G22,"")</f>
-        <v>0.092</v>
+        <v>0.0908</v>
       </c>
       <c r="I22" s="23">
-        <v>18200</v>
+        <v>17460</v>
       </c>
       <c r="J22" s="23"/>
       <c r="K22" s="24">
         <f>IFERROR(IF(OR(J22&gt;=L22,F22&gt;=L22),USD_CHF*LOOKUP(IF(J22="",F22,J22),{0,1,10,100,1000,2500,10000,20000,50000,100000},{0.0,0.091,0.032,0.02,0.017,0.015,0.012,0.011,0.009,0.008}),"MOQ="&amp;L22),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L22" s="23">
         <v>1</v>
       </c>
       <c r="M22" s="25">
         <f>IFERROR(IF(J22="",F22,J22)*K22,"")</f>
-        <v>0.1029</v>
+        <v>0.1031</v>
       </c>
       <c r="N22" s="23" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="O22" s="23">
         <v>155156</v>
@@ -17727,15 +17727,15 @@
       </c>
       <c r="V22" s="23"/>
       <c r="W22" s="24">
-        <f>IFERROR(IF(OR(V22&gt;=X22,F22&gt;=X22),LOOKUP(IF(V22="",F22,V22),{0,1,10,50,100,1000,2500,10000,50000,70000,100000},{0.0,0.092,0.035,0.0267,0.0239,0.0167,0.0145,0.0118,0.0094,0.0089,0.0085}),"MOQ="&amp;X22),"")</f>
-        <v>0.092</v>
+        <f>IFERROR(IF(OR(V22&gt;=X22,F22&gt;=X22),LOOKUP(IF(V22="",F22,V22),{0,1,10,50,100,1000,2500,10000,50000,70000,100000},{0.0,0.0908,0.0345,0.0263,0.0236,0.0164,0.0143,0.0117,0.0092,0.0088,0.0084}),"MOQ="&amp;X22),"")</f>
+        <v>0.0908</v>
       </c>
       <c r="X22" s="23">
         <v>1</v>
       </c>
       <c r="Y22" s="25">
         <f>IFERROR(IF(V22="",F22,V22)*W22,"")</f>
-        <v>0.092</v>
+        <v>0.0908</v>
       </c>
       <c r="Z22" s="23" t="s">
         <v>117</v>
@@ -17775,20 +17775,20 @@
       <c r="J23" s="23"/>
       <c r="K23" s="24">
         <f>IFERROR(IF(OR(J23&gt;=L23,F23&gt;=L23),USD_CHF*LOOKUP(IF(J23="",F23,J23),{0,1,10,100,1000,2000,10000,24000,50000},{0.0,0.671,0.307,0.217,0.198,0.166,0.151,0.15,0.142}),"MOQ="&amp;L23),"")</f>
-        <v>0.7586279169342752</v>
+        <v>0.7599468474284486</v>
       </c>
       <c r="L23" s="23">
         <v>1</v>
       </c>
       <c r="M23" s="25">
         <f>IFERROR(IF(J23="",F23,J23)*K23,"")</f>
-        <v>5.3104</v>
+        <v>5.3196</v>
       </c>
       <c r="N23" s="23" t="s">
         <v>125</v>
       </c>
       <c r="O23" s="23">
-        <v>11461</v>
+        <v>11401</v>
       </c>
       <c r="P23" s="23"/>
       <c r="Q23" s="24">
@@ -17828,11 +17828,11 @@
       </c>
       <c r="G24" s="24">
         <f>IF(MIN(Q24,K24,W24)&lt;&gt;0,MIN(Q24,K24,W24),"")</f>
-        <v>0.2454</v>
+        <v>0.2422</v>
       </c>
       <c r="H24" s="25">
         <f>IF(AND(ISNUMBER(F24),ISNUMBER(G24)),F24*G24,"")</f>
-        <v>0.7362</v>
+        <v>0.7266</v>
       </c>
       <c r="I24" s="23">
         <v>80</v>
@@ -17840,20 +17840,20 @@
       <c r="J24" s="23"/>
       <c r="K24" s="24">
         <f>IFERROR(IF(OR(J24&gt;=L24,F24&gt;=L24),USD_CHF*LOOKUP(IF(J24="",F24,J24),{0,1,10,100,1000,2500,10000,20000,50000,100000},{0.0,0.245,0.1,0.066,0.058,0.049,0.045,0.04,0.037,0.035}),"MOQ="&amp;L24),"")</f>
-        <v>0.27699529008777557</v>
+        <v>0.27747686679578226</v>
       </c>
       <c r="L24" s="23">
         <v>1</v>
       </c>
       <c r="M24" s="25">
         <f>IFERROR(IF(J24="",F24,J24)*K24,"")</f>
-        <v>0.831</v>
+        <v>0.8324</v>
       </c>
       <c r="N24" s="23" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="O24" s="23">
-        <v>21592</v>
+        <v>40182</v>
       </c>
       <c r="P24" s="23"/>
       <c r="Q24" s="24">
@@ -17871,19 +17871,19 @@
         <v>133</v>
       </c>
       <c r="U24" s="23">
-        <v>8737</v>
+        <v>8437</v>
       </c>
       <c r="V24" s="23"/>
       <c r="W24" s="24">
-        <f>IFERROR(IF(OR(V24&gt;=X24,F24&gt;=X24),LOOKUP(IF(V24="",F24,V24),{0,1,10,50,100,1000,2500,10000,20000,50000,100000},{0.0,0.2454,0.1048,0.0825,0.0752,0.0569,0.0516,0.0451,0.0425,0.0395,0.0376}),"MOQ="&amp;X24),"")</f>
-        <v>0.2454</v>
+        <f>IFERROR(IF(OR(V24&gt;=X24,F24&gt;=X24),LOOKUP(IF(V24="",F24,V24),{0,1,10,50,100,1000,2500,10000,20000,50000,100000},{0.0,0.2422,0.1034,0.0815,0.0742,0.0562,0.051,0.0446,0.042,0.039,0.0371}),"MOQ="&amp;X24),"")</f>
+        <v>0.2422</v>
       </c>
       <c r="X24" s="23">
         <v>1</v>
       </c>
       <c r="Y24" s="25">
         <f>IFERROR(IF(V24="",F24,V24)*W24,"")</f>
-        <v>0.7362</v>
+        <v>0.7266</v>
       </c>
       <c r="Z24" s="23" t="s">
         <v>134</v>
@@ -17911,32 +17911,32 @@
       </c>
       <c r="G25" s="24">
         <f>IF(MIN(Q25,K25,W25)&lt;&gt;0,MIN(Q25,K25,W25),"")</f>
-        <v>0.879</v>
+        <v>0.868</v>
       </c>
       <c r="H25" s="25">
         <f>IF(AND(ISNUMBER(F25),ISNUMBER(G25)),F25*G25,"")</f>
-        <v>3.516</v>
+        <v>3.472</v>
       </c>
       <c r="I25" s="23">
-        <v>18868</v>
+        <v>18768</v>
       </c>
       <c r="J25" s="23"/>
       <c r="K25" s="24">
-        <f>IFERROR(IF(OR(J25&gt;=L25,F25&gt;=L25),USD_CHF*LOOKUP(IF(J25="",F25,J25),{0,1,10,100,500,1000,2000,10000},{0.0,0.871,0.405,0.359,0.291,0.265,0.226,0.204}),"MOQ="&amp;L25),"")</f>
-        <v>0.9847465210875613</v>
+        <f>IFERROR(IF(OR(J25&gt;=L25,F25&gt;=L25),USD_CHF*LOOKUP(IF(J25="",F25,J25),{0,1,10,100,500,1000,2000,10000},{0.0,0.871,0.405,0.359,0.291,0.265,0.226,0.207}),"MOQ="&amp;L25),"")</f>
+        <v>0.9864585754250055</v>
       </c>
       <c r="L25" s="23">
         <v>1</v>
       </c>
       <c r="M25" s="25">
         <f>IFERROR(IF(J25="",F25,J25)*K25,"")</f>
-        <v>3.939</v>
+        <v>3.9458</v>
       </c>
       <c r="N25" s="23" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="O25" s="23">
-        <v>22022</v>
+        <v>22002</v>
       </c>
       <c r="P25" s="23"/>
       <c r="Q25" s="24">
@@ -17958,15 +17958,15 @@
       </c>
       <c r="V25" s="23"/>
       <c r="W25" s="24">
-        <f>IFERROR(IF(OR(V25&gt;=X25,F25&gt;=X25),LOOKUP(IF(V25="",F25,V25),{0,1,5,10,50,100,250,500,1000,2000},{0.0,0.879,0.49,0.454,0.379,0.347,0.306,0.275,0.244,0.213}),"MOQ="&amp;X25),"")</f>
-        <v>0.879</v>
+        <f>IFERROR(IF(OR(V25&gt;=X25,F25&gt;=X25),LOOKUP(IF(V25="",F25,V25),{0,1,5,10,50,100,250,500,1000,2000},{0.0,0.868,0.484,0.448,0.374,0.343,0.302,0.272,0.241,0.21}),"MOQ="&amp;X25),"")</f>
+        <v>0.868</v>
       </c>
       <c r="X25" s="23">
         <v>1</v>
       </c>
       <c r="Y25" s="25">
         <f>IFERROR(IF(V25="",F25,V25)*W25,"")</f>
-        <v>3.516</v>
+        <v>3.472</v>
       </c>
       <c r="Z25" s="23" t="s">
         <v>141</v>
@@ -17994,32 +17994,32 @@
       </c>
       <c r="G26" s="24">
         <f>IF(MIN(Q26,K26,W26)&lt;&gt;0,MIN(Q26,K26,W26),"")</f>
-        <v>0.379</v>
+        <v>0.374</v>
       </c>
       <c r="H26" s="25">
         <f>IF(AND(ISNUMBER(F26),ISNUMBER(G26)),F26*G26,"")</f>
-        <v>18.95</v>
+        <v>18.7</v>
       </c>
       <c r="I26" s="23">
-        <v>18868</v>
+        <v>18768</v>
       </c>
       <c r="J26" s="23"/>
       <c r="K26" s="24">
-        <f>IFERROR(IF(OR(J26&gt;=L26,F26&gt;=L26),USD_CHF*LOOKUP(IF(J26="",F26,J26),{0,1,10,100,500,1000,2000,10000},{0.0,0.871,0.405,0.359,0.291,0.265,0.226,0.204}),"MOQ="&amp;L26),"")</f>
-        <v>0.45789017341040456</v>
+        <f>IFERROR(IF(OR(J26&gt;=L26,F26&gt;=L26),USD_CHF*LOOKUP(IF(J26="",F26,J26),{0,1,10,100,500,1000,2000,10000},{0.0,0.871,0.405,0.359,0.291,0.265,0.226,0.207}),"MOQ="&amp;L26),"")</f>
+        <v>0.45868624919302786</v>
       </c>
       <c r="L26" s="23">
         <v>1</v>
       </c>
       <c r="M26" s="25">
         <f>IFERROR(IF(J26="",F26,J26)*K26,"")</f>
-        <v>22.8945</v>
+        <v>22.9343</v>
       </c>
       <c r="N26" s="23" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="O26" s="23">
-        <v>22022</v>
+        <v>22002</v>
       </c>
       <c r="P26" s="23"/>
       <c r="Q26" s="24">
@@ -18041,15 +18041,15 @@
       </c>
       <c r="V26" s="23"/>
       <c r="W26" s="24">
-        <f>IFERROR(IF(OR(V26&gt;=X26,F26&gt;=X26),LOOKUP(IF(V26="",F26,V26),{0,1,5,10,50,100,250,500,1000,2000},{0.0,0.879,0.49,0.454,0.379,0.347,0.306,0.275,0.244,0.213}),"MOQ="&amp;X26),"")</f>
-        <v>0.379</v>
+        <f>IFERROR(IF(OR(V26&gt;=X26,F26&gt;=X26),LOOKUP(IF(V26="",F26,V26),{0,1,5,10,50,100,250,500,1000,2000},{0.0,0.868,0.484,0.448,0.374,0.343,0.302,0.272,0.241,0.21}),"MOQ="&amp;X26),"")</f>
+        <v>0.374</v>
       </c>
       <c r="X26" s="23">
         <v>1</v>
       </c>
       <c r="Y26" s="25">
         <f>IFERROR(IF(V26="",F26,V26)*W26,"")</f>
-        <v>18.95</v>
+        <v>18.7</v>
       </c>
       <c r="Z26" s="23" t="s">
         <v>141</v>
@@ -18077,32 +18077,32 @@
       </c>
       <c r="G27" s="24">
         <f>IF(MIN(Q27,K27,W27)&lt;&gt;0,MIN(Q27,K27,W27),"")</f>
-        <v>0.30752130164846925</v>
+        <v>0.30805595007531744</v>
       </c>
       <c r="H27" s="25">
         <f>IF(AND(ISNUMBER(F27),ISNUMBER(G27)),F27*G27,"")</f>
-        <v>0.3075</v>
+        <v>0.3081</v>
       </c>
       <c r="I27" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J27" s="23"/>
       <c r="K27" s="24">
         <f>IFERROR(IF(OR(J27&gt;=L27,F27&gt;=L27),USD_CHF*LOOKUP(IF(J27="",F27,J27),{0,1,10,100,1000,2500,10000,20000,50000,100000},{0.0,0.272,0.115,0.077,0.068,0.058,0.049,0.047,0.045,0.042}),"MOQ="&amp;L27),"")</f>
-        <v>0.30752130164846925</v>
+        <v>0.30805595007531744</v>
       </c>
       <c r="L27" s="23">
         <v>1</v>
       </c>
       <c r="M27" s="25">
         <f>IFERROR(IF(J27="",F27,J27)*K27,"")</f>
-        <v>0.3075</v>
+        <v>0.3081</v>
       </c>
       <c r="N27" s="23" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="O27" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="P27" s="23"/>
       <c r="Q27" s="24">
@@ -18149,25 +18149,25 @@
         <v>0.68</v>
       </c>
       <c r="I28" s="23">
-        <v>140098</v>
+        <v>135928</v>
       </c>
       <c r="J28" s="23"/>
       <c r="K28" s="24">
         <f>IFERROR(IF(OR(J28&gt;=L28,F28&gt;=L28),USD_CHF*LOOKUP(IF(J28="",F28,J28),{0,1,10,100,1000,3000,9000,24000,45000},{0.0,0.308,0.129,0.087,0.077,0.066,0.059,0.055,0.052}),"MOQ="&amp;L28),"")</f>
-        <v>0.34822265039606076</v>
+        <v>0.34882806111469766</v>
       </c>
       <c r="L28" s="23">
         <v>1</v>
       </c>
       <c r="M28" s="25">
         <f>IFERROR(IF(J28="",F28,J28)*K28,"")</f>
-        <v>0.6964</v>
+        <v>0.6977</v>
       </c>
       <c r="N28" s="23" t="s">
         <v>600</v>
       </c>
       <c r="O28" s="23">
-        <v>41679</v>
+        <v>38599</v>
       </c>
       <c r="P28" s="23"/>
       <c r="Q28" s="24">
@@ -18185,19 +18185,19 @@
         <v>160</v>
       </c>
       <c r="U28" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V28" s="23"/>
       <c r="W28" s="24">
-        <f>IFERROR(IF(OR(V28&gt;=X28,F28&gt;=X28),LOOKUP(IF(V28="",F28,V28),{0,1,10,50,100,500,1000,3000,15000,75000},{0.0,0.355,0.234,0.158,0.135,0.098,0.088,0.076,0.066,0.063}),"MOQ="&amp;X28),"")</f>
-        <v>0.355</v>
+        <f>IFERROR(IF(OR(V28&gt;=X28,F28&gt;=X28),LOOKUP(IF(V28="",F28,V28),{0,1,10,50,100,500,1000,3000,15000,75000},{0.0,0.351,0.231,0.156,0.133,0.096,0.087,0.075,0.065,0.062}),"MOQ="&amp;X28),"")</f>
+        <v>0.351</v>
       </c>
       <c r="X28" s="23">
         <v>1</v>
       </c>
       <c r="Y28" s="25">
         <f>IFERROR(IF(V28="",F28,V28)*W28,"")</f>
-        <v>0.71</v>
+        <v>0.702</v>
       </c>
       <c r="Z28" s="23" t="s">
         <v>161</v>
@@ -18225,32 +18225,32 @@
       </c>
       <c r="G29" s="24">
         <f>IF(MIN(Q29,K29,W29)&lt;&gt;0,MIN(Q29,K29,W29),"")</f>
-        <v>1.6280539499036606</v>
+        <v>1.63088444157521</v>
       </c>
       <c r="H29" s="25">
         <f>IF(AND(ISNUMBER(F29),ISNUMBER(G29)),F29*G29,"")</f>
-        <v>3.2561</v>
+        <v>3.2618</v>
       </c>
       <c r="I29" s="23">
-        <v>2614</v>
+        <v>2414</v>
       </c>
       <c r="J29" s="23"/>
       <c r="K29" s="24">
         <f>IFERROR(IF(OR(J29&gt;=L29,F29&gt;=L29),USD_CHF*LOOKUP(IF(J29="",F29,J29),{0,1,10,100,500,1000,2000},{0.0,1.44,0.814,0.747,0.593,0.549,0.528}),"MOQ="&amp;L29),"")</f>
-        <v>1.6280539499036606</v>
+        <v>1.63088444157521</v>
       </c>
       <c r="L29" s="23">
         <v>1</v>
       </c>
       <c r="M29" s="25">
         <f>IFERROR(IF(J29="",F29,J29)*K29,"")</f>
-        <v>3.2561</v>
+        <v>3.2618</v>
       </c>
       <c r="N29" s="23" t="s">
         <v>601</v>
       </c>
       <c r="O29" s="23">
-        <v>3110</v>
+        <v>3107</v>
       </c>
       <c r="P29" s="23"/>
       <c r="Q29" s="24">
@@ -18268,11 +18268,11 @@
         <v>168</v>
       </c>
       <c r="U29" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V29" s="23"/>
       <c r="W29" s="24">
-        <f>IFERROR(IF(OR(V29&gt;=X29,F29&gt;=X29),LOOKUP(IF(V29="",F29,V29),{0,1,1000,7000},{0.0,0.542,0.542,0.516}),"MOQ="&amp;X29),"")</f>
+        <f>IFERROR(IF(OR(V29&gt;=X29,F29&gt;=X29),LOOKUP(IF(V29="",F29,V29),{0,1,1000,7000},{0.0,0.543,0.543,0.515}),"MOQ="&amp;X29),"")</f>
         <v/>
       </c>
       <c r="X29" s="23">
@@ -18308,32 +18308,32 @@
       </c>
       <c r="G30" s="24">
         <f>IF(MIN(Q30,K30,W30)&lt;&gt;0,MIN(Q30,K30,W30),"")</f>
-        <v>0.326</v>
+        <v>0.322</v>
       </c>
       <c r="H30" s="25">
         <f>IF(AND(ISNUMBER(F30),ISNUMBER(G30)),F30*G30,"")</f>
-        <v>0.652</v>
+        <v>0.644</v>
       </c>
       <c r="I30" s="23">
-        <v>41033</v>
+        <v>21268</v>
       </c>
       <c r="J30" s="23"/>
       <c r="K30" s="24">
-        <f>IFERROR(IF(OR(J30&gt;=L30,F30&gt;=L30),USD_CHF*LOOKUP(IF(J30="",F30,J30),{0,1,10,100,1000,3000,9000,24000,45000,99000},{0.0,0.363,0.153,0.104,0.095,0.076,0.068,0.065,0.061,0.059}),"MOQ="&amp;L30),"")</f>
-        <v>0.4104052665382144</v>
+        <f>IFERROR(IF(OR(J30&gt;=L30,F30&gt;=L30),USD_CHF*LOOKUP(IF(J30="",F30,J30),{0,1,10,100,1000,3000,9000,45000,99000},{0.0,0.371,0.158,0.108,0.098,0.081,0.079,0.061,0.059}),"MOQ="&amp;L30),"")</f>
+        <v>0.4201792554336131</v>
       </c>
       <c r="L30" s="23">
         <v>1</v>
       </c>
       <c r="M30" s="25">
         <f>IFERROR(IF(J30="",F30,J30)*K30,"")</f>
-        <v>0.8208</v>
+        <v>0.8404</v>
       </c>
       <c r="N30" s="23" t="s">
         <v>602</v>
       </c>
       <c r="O30" s="23">
-        <v>51663</v>
+        <v>51512</v>
       </c>
       <c r="P30" s="23"/>
       <c r="Q30" s="24">
@@ -18351,19 +18351,19 @@
         <v>175</v>
       </c>
       <c r="U30" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V30" s="23"/>
       <c r="W30" s="24">
-        <f>IFERROR(IF(OR(V30&gt;=X30,F30&gt;=X30),LOOKUP(IF(V30="",F30,V30),{0,1,5,10,50,100,1000,3000,6000,9000,45000},{0.0,0.326,0.229,0.187,0.122,0.105,0.079,0.075,0.073,0.072,0.07}),"MOQ="&amp;X30),"")</f>
-        <v>0.326</v>
+        <f>IFERROR(IF(OR(V30&gt;=X30,F30&gt;=X30),LOOKUP(IF(V30="",F30,V30),{0,1,5,10,50,100,1000,3000,6000,9000,45000},{0.0,0.322,0.226,0.185,0.12,0.104,0.078,0.074,0.072,0.071,0.069}),"MOQ="&amp;X30),"")</f>
+        <v>0.322</v>
       </c>
       <c r="X30" s="23">
         <v>1</v>
       </c>
       <c r="Y30" s="25">
         <f>IFERROR(IF(V30="",F30,V30)*W30,"")</f>
-        <v>0.652</v>
+        <v>0.644</v>
       </c>
       <c r="Z30" s="23" t="s">
         <v>176</v>
@@ -18398,14 +18398,14 @@
         <v>1.146</v>
       </c>
       <c r="I31" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J31" s="23"/>
       <c r="N31" s="23" t="s">
         <v>603</v>
       </c>
       <c r="O31" s="23">
-        <v>31438</v>
+        <v>30938</v>
       </c>
       <c r="P31" s="23"/>
       <c r="Q31" s="24">
@@ -18475,20 +18475,20 @@
       <c r="J32" s="23"/>
       <c r="K32" s="24">
         <f>IFERROR(IF(OR(J32&gt;=L32,F32&gt;=L32),USD_CHF*LOOKUP(IF(J32="",F32,J32),{0,1,10,100,1000,3000,9000,24000,45000},{0.0,0.254,0.167,0.084,0.067,0.052,0.045,0.043,0.041}),"MOQ="&amp;L32),"")</f>
-        <v>0.188809034467994</v>
+        <v>0.18913729287712505</v>
       </c>
       <c r="L32" s="23">
         <v>1</v>
       </c>
       <c r="M32" s="25">
         <f>IFERROR(IF(J32="",F32,J32)*K32,"")</f>
-        <v>2.8321</v>
+        <v>2.8371</v>
       </c>
       <c r="N32" s="23" t="s">
         <v>604</v>
       </c>
       <c r="O32" s="23">
-        <v>42223</v>
+        <v>41920</v>
       </c>
       <c r="P32" s="23"/>
       <c r="Q32" s="24">
@@ -18510,7 +18510,7 @@
       </c>
       <c r="V32" s="23"/>
       <c r="W32" s="24">
-        <f>IFERROR(IF(OR(V32&gt;=X32,F32&gt;=X32),LOOKUP(IF(V32="",F32,V32),{0,1,10,50,100,1000,2500,3000,6000,9000,45000},{0.0,0.28,0.184,0.1448,0.0955,0.0848,0.0704,0.0669,0.0622,0.0575,0.0562}),"MOQ="&amp;X32),"")</f>
+        <f>IFERROR(IF(OR(V32&gt;=X32,F32&gt;=X32),LOOKUP(IF(V32="",F32,V32),{0,1,10,50,100,1000,2500,3000,6000,9000,45000},{0.0,0.28,0.184,0.1448,0.0955,0.0848,0.0705,0.0669,0.0623,0.0575,0.0562}),"MOQ="&amp;X32),"")</f>
         <v>0.184</v>
       </c>
       <c r="X32" s="23">
@@ -18553,25 +18553,25 @@
         <v>3.0</v>
       </c>
       <c r="I33" s="23">
-        <v>42722</v>
+        <v>40692</v>
       </c>
       <c r="J33" s="23"/>
       <c r="K33" s="24">
         <f>IFERROR(IF(OR(J33&gt;=L33,F33&gt;=L33),USD_CHF*LOOKUP(IF(J33="",F33,J33),{0,1,10,100,500,1000,3000,6000},{0.0,1.37,1.04,0.736,0.6,0.598,0.552,0.531}),"MOQ="&amp;L33),"")</f>
-        <v>1.5489124384500106</v>
+        <v>1.551605336776415</v>
       </c>
       <c r="L33" s="23">
         <v>1</v>
       </c>
       <c r="M33" s="25">
         <f>IFERROR(IF(J33="",F33,J33)*K33,"")</f>
-        <v>3.0978</v>
+        <v>3.1032</v>
       </c>
       <c r="N33" s="23" t="s">
         <v>605</v>
       </c>
       <c r="O33" s="23">
-        <v>36451</v>
+        <v>35896</v>
       </c>
       <c r="P33" s="23"/>
       <c r="Q33" s="24">
@@ -18589,11 +18589,11 @@
         <v>198</v>
       </c>
       <c r="U33" s="23">
-        <v>17096</v>
+        <v>16840</v>
       </c>
       <c r="V33" s="23"/>
       <c r="W33" s="24">
-        <f>IFERROR(IF(OR(V33&gt;=X33,F33&gt;=X33),LOOKUP(IF(V33="",F33,V33),{0,1,10,100,500,1000,1500,3000,6000},{0.0,1.84,0.841,0.641,0.551,0.522,0.506,0.484,0.463}),"MOQ="&amp;X33),"")</f>
+        <f>IFERROR(IF(OR(V33&gt;=X33,F33&gt;=X33),LOOKUP(IF(V33="",F33,V33),{0,1,10,100,500,1000,1500,3000,6000},{0.0,1.84,0.841,0.641,0.552,0.523,0.507,0.484,0.463}),"MOQ="&amp;X33),"")</f>
         <v>1.84</v>
       </c>
       <c r="X33" s="23">
@@ -18629,26 +18629,26 @@
       </c>
       <c r="G34" s="24">
         <f>IF(MIN(Q34,K34,W34)&lt;&gt;0,MIN(Q34,K34,W34),"")</f>
-        <v>1.0864998929565401</v>
+        <v>1.088388853023456</v>
       </c>
       <c r="H34" s="25">
         <f>IF(AND(ISNUMBER(F34),ISNUMBER(G34)),F34*G34,"")</f>
-        <v>1.0865</v>
+        <v>1.0884</v>
       </c>
       <c r="I34" s="23">
-        <v>13265</v>
+        <v>13255</v>
       </c>
       <c r="J34" s="23"/>
       <c r="K34" s="24">
         <f>IFERROR(IF(OR(J34&gt;=L34,F34&gt;=L34),USD_CHF*LOOKUP(IF(J34="",F34,J34),{0,1,10,100,500,1000,3000,24000},{0.0,0.961,0.628,0.467,0.432,0.371,0.371,0.343}),"MOQ="&amp;L34),"")</f>
-        <v>1.0864998929565401</v>
+        <v>1.088388853023456</v>
       </c>
       <c r="L34" s="23">
         <v>1</v>
       </c>
       <c r="M34" s="25">
         <f>IFERROR(IF(J34="",F34,J34)*K34,"")</f>
-        <v>1.0865</v>
+        <v>1.0884</v>
       </c>
       <c r="N34" s="23" t="s">
         <v>606</v>
@@ -18701,19 +18701,19 @@
         <v>0.48</v>
       </c>
       <c r="I35" s="23">
-        <v>11191</v>
+        <v>11091</v>
       </c>
       <c r="J35" s="23"/>
       <c r="K35" s="24">
         <f>IFERROR(IF(OR(J35&gt;=L35,F35&gt;=L35),USD_CHF*LOOKUP(IF(J35="",F35,J35),{0,1,10,100,1000,3000,9000,24000,45000},{0.0,0.217,0.149,0.077,0.069,0.054,0.049,0.044,0.041}),"MOQ="&amp;L35),"")</f>
-        <v>0.24533868550631552</v>
+        <v>0.2457652248762643</v>
       </c>
       <c r="L35" s="23">
         <v>1</v>
       </c>
       <c r="M35" s="25">
         <f>IFERROR(IF(J35="",F35,J35)*K35,"")</f>
-        <v>0.4907</v>
+        <v>0.4915</v>
       </c>
       <c r="N35" s="23" t="s">
         <v>607</v>
@@ -18771,14 +18771,14 @@
       <c r="J36" s="23"/>
       <c r="K36" s="24">
         <f>IFERROR(IF(OR(J36&gt;=L36,F36&gt;=L36),USD_CHF*LOOKUP(IF(J36="",F36,J36),{0,1,10,100,500,1000,4000,8000,24000},{0.0,0.499,0.347,0.215,0.173,0.128,0.122,0.102,0.1}),"MOQ="&amp;L36),"")</f>
-        <v>0.564165917362449</v>
+        <v>0.5651467613514096</v>
       </c>
       <c r="L36" s="23">
         <v>1</v>
       </c>
       <c r="M36" s="25">
         <f>IFERROR(IF(J36="",F36,J36)*K36,"")</f>
-        <v>1.1283</v>
+        <v>1.1303</v>
       </c>
       <c r="N36" s="23" t="s">
         <v>608</v>
@@ -18836,14 +18836,14 @@
       <c r="J37" s="23"/>
       <c r="K37" s="24">
         <f>IFERROR(IF(OR(J37&gt;=L37,F37&gt;=L37),USD_CHF*LOOKUP(IF(J37="",F37,J37),{0,1,10,100,500,1000,2000,4000,8000},{0.0,0.435,0.301,0.204,0.16,0.145,0.133,0.121,0.106}),"MOQ="&amp;L37),"")</f>
-        <v>0.4918079640333975</v>
+        <v>0.49266300839251137</v>
       </c>
       <c r="L37" s="23">
         <v>1</v>
       </c>
       <c r="M37" s="25">
         <f>IFERROR(IF(J37="",F37,J37)*K37,"")</f>
-        <v>0.9836</v>
+        <v>0.9853</v>
       </c>
       <c r="N37" s="23" t="s">
         <v>609</v>
@@ -18901,14 +18901,14 @@
       <c r="J38" s="23"/>
       <c r="K38" s="24">
         <f>IFERROR(IF(OR(J38&gt;=L38,F38&gt;=L38),USD_CHF*LOOKUP(IF(J38="",F38,J38),{0,1,10,100,750,2250,9750},{0.0,0.344,0.234,0.11,0.087,0.085,0.084}),"MOQ="&amp;L38),"")</f>
-        <v>0.3889239991436522</v>
+        <v>0.38960017215407794</v>
       </c>
       <c r="L38" s="23">
         <v>1</v>
       </c>
       <c r="M38" s="25">
         <f>IFERROR(IF(J38="",F38,J38)*K38,"")</f>
-        <v>0.7778</v>
+        <v>0.7792</v>
       </c>
       <c r="N38" s="23" t="s">
         <v>610</v>
@@ -18932,11 +18932,11 @@
         <v>236</v>
       </c>
       <c r="U38" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V38" s="23"/>
       <c r="W38" s="24">
-        <f>IFERROR(IF(OR(V38&gt;=X38,F38&gt;=X38),LOOKUP(IF(V38="",F38,V38),{0,1,10,100,500,750,1500,2250},{0.0,0.38,0.284,0.193,0.142,0.131,0.112,0.103}),"MOQ="&amp;X38),"")</f>
+        <f>IFERROR(IF(OR(V38&gt;=X38,F38&gt;=X38),LOOKUP(IF(V38="",F38,V38),{0,1,10,100,500,750,1500,2250},{0.0,0.38,0.284,0.193,0.143,0.131,0.112,0.103}),"MOQ="&amp;X38),"")</f>
         <v>0.38</v>
       </c>
       <c r="X38" s="23">
@@ -18972,11 +18972,11 @@
       </c>
       <c r="G39" s="24">
         <f>IF(MIN(Q39,K39,W39)&lt;&gt;0,MIN(Q39,K39,W39),"")</f>
-        <v>0.5438152429886532</v>
+        <v>0.5447607058317194</v>
       </c>
       <c r="H39" s="25">
         <f>IF(AND(ISNUMBER(F39),ISNUMBER(G39)),F39*G39,"")</f>
-        <v>0.5438</v>
+        <v>0.5448</v>
       </c>
       <c r="I39" s="23">
         <v>4669</v>
@@ -18984,14 +18984,14 @@
       <c r="J39" s="23"/>
       <c r="K39" s="24">
         <f>IFERROR(IF(OR(J39&gt;=L39,F39&gt;=L39),USD_CHF*LOOKUP(IF(J39="",F39,J39),{0,1,10,100,1000,3000,9000,24000},{0.0,0.481,0.332,0.192,0.176,0.147,0.144,0.135}),"MOQ="&amp;L39),"")</f>
-        <v>0.5438152429886532</v>
+        <v>0.5447607058317194</v>
       </c>
       <c r="L39" s="23">
         <v>1</v>
       </c>
       <c r="M39" s="25">
         <f>IFERROR(IF(J39="",F39,J39)*K39,"")</f>
-        <v>0.5438</v>
+        <v>0.5448</v>
       </c>
       <c r="N39" s="23" t="s">
         <v>611</v>
@@ -19051,25 +19051,25 @@
         <v>0.92</v>
       </c>
       <c r="I40" s="23">
-        <v>20355</v>
+        <v>20255</v>
       </c>
       <c r="J40" s="23"/>
       <c r="K40" s="24">
         <f>IFERROR(IF(OR(J40&gt;=L40,F40&gt;=L40),USD_CHF*LOOKUP(IF(J40="",F40,J40),{0,1,50,100,500,1000,2500,4000},{0.0,0.209,0.203,0.187,0.178,0.162,0.137,0.137}),"MOQ="&amp;L40),"")</f>
-        <v>0.23629394134018405</v>
+        <v>0.23670475575640199</v>
       </c>
       <c r="L40" s="23">
         <v>1</v>
       </c>
       <c r="M40" s="25">
         <f>IFERROR(IF(J40="",F40,J40)*K40,"")</f>
-        <v>0.9452</v>
+        <v>0.9468</v>
       </c>
       <c r="N40" s="23" t="s">
         <v>612</v>
       </c>
       <c r="O40" s="23">
-        <v>28136</v>
+        <v>28106</v>
       </c>
       <c r="P40" s="23"/>
       <c r="Q40" s="24">
@@ -19109,11 +19109,11 @@
       </c>
       <c r="G41" s="24">
         <f>IF(MIN(Q41,K41,W41)&lt;&gt;0,MIN(Q41,K41,W41),"")</f>
-        <v>2.114208948833226</v>
+        <v>2.1178846567678073</v>
       </c>
       <c r="H41" s="25">
         <f>IF(AND(ISNUMBER(F41),ISNUMBER(G41)),F41*G41,"")</f>
-        <v>4.2284</v>
+        <v>4.2358</v>
       </c>
       <c r="I41" s="23">
         <v>916</v>
@@ -19121,14 +19121,14 @@
       <c r="J41" s="23"/>
       <c r="K41" s="24">
         <f>IFERROR(IF(OR(J41&gt;=L41,F41&gt;=L41),USD_CHF*LOOKUP(IF(J41="",F41,J41),{0,1,10,100,500},{0.0,1.87,1.65,1.37,1.37}),"MOQ="&amp;L41),"")</f>
-        <v>2.114208948833226</v>
+        <v>2.1178846567678073</v>
       </c>
       <c r="L41" s="23">
         <v>1</v>
       </c>
       <c r="M41" s="25">
         <f>IFERROR(IF(J41="",F41,J41)*K41,"")</f>
-        <v>4.2284</v>
+        <v>4.2358</v>
       </c>
       <c r="N41" s="23" t="s">
         <v>613</v>
@@ -19181,14 +19181,14 @@
         <v>1.38</v>
       </c>
       <c r="I42" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J42" s="23"/>
       <c r="N42" s="23" t="s">
         <v>603</v>
       </c>
       <c r="O42" s="23">
-        <v>62562</v>
+        <v>60443</v>
       </c>
       <c r="P42" s="23"/>
       <c r="Q42" s="24">
@@ -19210,7 +19210,7 @@
       </c>
       <c r="V42" s="23"/>
       <c r="W42" s="24">
-        <f>IFERROR(IF(OR(V42&gt;=X42,F42&gt;=X42),LOOKUP(IF(V42="",F42,V42),{0,1,5,20,100,500},{0.0,0.296,0.296,0.253,0.212,0.17}),"MOQ="&amp;X42),"")</f>
+        <f>IFERROR(IF(OR(V42&gt;=X42,F42&gt;=X42),LOOKUP(IF(V42="",F42,V42),{0,1,5,20,100,500},{0.0,0.297,0.297,0.254,0.212,0.17}),"MOQ="&amp;X42),"")</f>
         <v/>
       </c>
       <c r="X42" s="23">
@@ -19253,14 +19253,14 @@
         <v>0.57</v>
       </c>
       <c r="I43" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J43" s="23"/>
       <c r="N43" s="23" t="s">
         <v>603</v>
       </c>
       <c r="O43" s="23">
-        <v>48009</v>
+        <v>47982</v>
       </c>
       <c r="P43" s="23"/>
       <c r="Q43" s="24">
@@ -19325,25 +19325,25 @@
         <v>0.5</v>
       </c>
       <c r="I44" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J44" s="23"/>
       <c r="K44" s="24">
         <f>IFERROR(IF(OR(J44&gt;=L44,F44&gt;=L44),USD_CHF*LOOKUP(IF(J44="",F44,J44),{0,1,10,100,500,1000,2500,5000,10000,25000},{0.0,0.607,0.462,0.359,0.3,0.275,0.25,0.227,0.209,0.202}),"MOQ="&amp;L44),"")</f>
-        <v>0.6862699636052236</v>
+        <v>0.6874630944695503</v>
       </c>
       <c r="L44" s="23">
         <v>1</v>
       </c>
       <c r="M44" s="25">
         <f>IFERROR(IF(J44="",F44,J44)*K44,"")</f>
-        <v>0.6863</v>
+        <v>0.6875</v>
       </c>
       <c r="N44" s="23" t="s">
         <v>614</v>
       </c>
       <c r="O44" s="23">
-        <v>22865</v>
+        <v>22323</v>
       </c>
       <c r="P44" s="23"/>
       <c r="Q44" s="24">
@@ -19365,7 +19365,7 @@
       </c>
       <c r="V44" s="23"/>
       <c r="W44" s="24">
-        <f>IFERROR(IF(OR(V44&gt;=X44,F44&gt;=X44),LOOKUP(IF(V44="",F44,V44),{0,1,10,100,500,1000},{0.0,0.819,0.715,0.616,0.513,0.409}),"MOQ="&amp;X44),"")</f>
+        <f>IFERROR(IF(OR(V44&gt;=X44,F44&gt;=X44),LOOKUP(IF(V44="",F44,V44),{0,1,10,100,500,1000},{0.0,0.819,0.716,0.616,0.513,0.41}),"MOQ="&amp;X44),"")</f>
         <v>0.819</v>
       </c>
       <c r="X44" s="23">
@@ -19408,14 +19408,14 @@
         <v>0.7</v>
       </c>
       <c r="I45" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J45" s="23"/>
       <c r="N45" s="23" t="s">
         <v>603</v>
       </c>
       <c r="O45" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="P45" s="23"/>
       <c r="Q45" s="24">
@@ -19462,14 +19462,14 @@
         <v>0.56</v>
       </c>
       <c r="I46" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J46" s="23"/>
       <c r="N46" s="23" t="s">
         <v>603</v>
       </c>
       <c r="O46" s="23">
-        <v>2636</v>
+        <v>2601</v>
       </c>
       <c r="P46" s="23"/>
       <c r="Q46" s="24">
@@ -19491,15 +19491,15 @@
       </c>
       <c r="V46" s="23"/>
       <c r="W46" s="24">
-        <f>IFERROR(IF(OR(V46&gt;=X46,F46&gt;=X46),LOOKUP(IF(V46="",F46,V46),{0,1,10,100,500,1000},{0.0,0.928,0.81,0.697,0.582,0.464}),"MOQ="&amp;X46),"")</f>
-        <v>0.928</v>
+        <f>IFERROR(IF(OR(V46&gt;=X46,F46&gt;=X46),LOOKUP(IF(V46="",F46,V46),{0,1,10,100,500,1000},{0.0,0.929,0.811,0.698,0.583,0.464}),"MOQ="&amp;X46),"")</f>
+        <v>0.929</v>
       </c>
       <c r="X46" s="23">
         <v>1</v>
       </c>
       <c r="Y46" s="25">
         <f>IFERROR(IF(V46="",F46,V46)*W46,"")</f>
-        <v>0.928</v>
+        <v>0.929</v>
       </c>
       <c r="Z46" s="23" t="s">
         <v>299</v>
@@ -19534,7 +19534,7 @@
         <v>1.08</v>
       </c>
       <c r="U47" s="23">
-        <v>8065</v>
+        <v>8035</v>
       </c>
       <c r="V47" s="23"/>
       <c r="W47" s="24">
@@ -19581,7 +19581,7 @@
         <v>1.08</v>
       </c>
       <c r="U48" s="23">
-        <v>11087</v>
+        <v>11077</v>
       </c>
       <c r="V48" s="23"/>
       <c r="W48" s="24">
@@ -19621,11 +19621,11 @@
       </c>
       <c r="G49" s="24">
         <f>IF(MIN(Q49,K49,W49)&lt;&gt;0,MIN(Q49,K49,W49),"")</f>
-        <v>1.5036887176193532</v>
+        <v>1.5063029911771038</v>
       </c>
       <c r="H49" s="25">
         <f>IF(AND(ISNUMBER(F49),ISNUMBER(G49)),F49*G49,"")</f>
-        <v>1.5037</v>
+        <v>1.5063</v>
       </c>
       <c r="I49" s="23">
         <v>1090</v>
@@ -19633,14 +19633,14 @@
       <c r="J49" s="23"/>
       <c r="K49" s="24">
         <f>IFERROR(IF(OR(J49&gt;=L49,F49&gt;=L49),USD_CHF*LOOKUP(IF(J49="",F49,J49),{0,1,250,500,1000},{0.0,1.33,1.1,0.8,0.681}),"MOQ="&amp;L49),"")</f>
-        <v>1.5036887176193532</v>
+        <v>1.5063029911771038</v>
       </c>
       <c r="L49" s="23">
         <v>1</v>
       </c>
       <c r="M49" s="25">
         <f>IFERROR(IF(J49="",F49,J49)*K49,"")</f>
-        <v>1.5037</v>
+        <v>1.5063</v>
       </c>
       <c r="N49" s="23" t="s">
         <v>324</v>
@@ -19675,25 +19675,25 @@
         <v>2.38</v>
       </c>
       <c r="I50" s="23">
-        <v>38725</v>
+        <v>38720</v>
       </c>
       <c r="J50" s="23"/>
       <c r="K50" s="24">
         <f>IFERROR(IF(OR(J50&gt;=L50,F50&gt;=L50),USD_CHF*LOOKUP(IF(J50="",F50,J50),{0,1,250,500,1000},{0.0,1.1,0.925,0.602,0.602}),"MOQ="&amp;L50),"")</f>
-        <v>1.2436523228430743</v>
+        <v>1.2458145039810633</v>
       </c>
       <c r="L50" s="23">
         <v>1</v>
       </c>
       <c r="M50" s="25">
         <f>IFERROR(IF(J50="",F50,J50)*K50,"")</f>
-        <v>2.4873</v>
+        <v>2.4916</v>
       </c>
       <c r="N50" s="23" t="s">
         <v>333</v>
       </c>
       <c r="O50" s="23">
-        <v>4763</v>
+        <v>10718</v>
       </c>
       <c r="P50" s="23"/>
       <c r="Q50" s="24">
@@ -19745,14 +19745,14 @@
       <c r="J51" s="23"/>
       <c r="K51" s="24">
         <f>IFERROR(IF(OR(J51&gt;=L51,F51&gt;=L51),USD_CHF*LOOKUP(IF(J51="",F51,J51),{0,1,10,100,1000,3000,9000,24000},{0.0,0.281,0.191,0.099,0.089,0.07,0.06,0.059}),"MOQ="&amp;L51),"")</f>
-        <v>0.31769663883536714</v>
+        <v>0.31824897783516254</v>
       </c>
       <c r="L51" s="23">
         <v>1</v>
       </c>
       <c r="M51" s="25">
         <f>IFERROR(IF(J51="",F51,J51)*K51,"")</f>
-        <v>0.9531</v>
+        <v>0.9547</v>
       </c>
       <c r="N51" s="23" t="s">
         <v>615</v>
@@ -19780,7 +19780,7 @@
       </c>
       <c r="V51" s="23"/>
       <c r="W51" s="24">
-        <f>IFERROR(IF(OR(V51&gt;=X51,F51&gt;=X51),LOOKUP(IF(V51="",F51,V51),{0,1,10,25,100,500,1000,3000,6000,30000,45000},{0.0,0.53,0.4,0.311,0.201,0.135,0.121,0.107,0.103,0.098,0.096}),"MOQ="&amp;X51),"")</f>
+        <f>IFERROR(IF(OR(V51&gt;=X51,F51&gt;=X51),LOOKUP(IF(V51="",F51,V51),{0,1,10,25,100,500,1000,3000,6000,30000,45000},{0.0,0.53,0.4,0.312,0.201,0.135,0.121,0.107,0.103,0.098,0.096}),"MOQ="&amp;X51),"")</f>
         <v>0.53</v>
       </c>
       <c r="X51" s="23">
@@ -19816,11 +19816,11 @@
       </c>
       <c r="G52" s="24">
         <f>IF(MIN(Q52,K52,W52)&lt;&gt;0,MIN(Q52,K52,W52),"")</f>
-        <v>3.1204367373153494</v>
+        <v>3.1258618463524854</v>
       </c>
       <c r="H52" s="25">
         <f>IF(AND(ISNUMBER(F52),ISNUMBER(G52)),F52*G52,"")</f>
-        <v>18.7226</v>
+        <v>18.7552</v>
       </c>
       <c r="I52" s="23">
         <v>10125</v>
@@ -19828,20 +19828,20 @@
       <c r="J52" s="23"/>
       <c r="K52" s="24">
         <f>IFERROR(IF(OR(J52&gt;=L52,F52&gt;=L52),USD_CHF*LOOKUP(IF(J52="",F52,J52),{0,1,10,50,100,500,1000,5000},{0.0,2.76,1.9,1.77,1.37,1.15,1.13,1.13}),"MOQ="&amp;L52),"")</f>
-        <v>3.1204367373153494</v>
+        <v>3.1258618463524854</v>
       </c>
       <c r="L52" s="23">
         <v>1</v>
       </c>
       <c r="M52" s="25">
         <f>IFERROR(IF(J52="",F52,J52)*K52,"")</f>
-        <v>18.7226</v>
+        <v>18.7552</v>
       </c>
       <c r="N52" s="23" t="s">
         <v>616</v>
       </c>
       <c r="O52" s="23">
-        <v>12460</v>
+        <v>12440</v>
       </c>
       <c r="P52" s="23"/>
       <c r="Q52" s="24">
@@ -19859,7 +19859,7 @@
         <v>348</v>
       </c>
       <c r="U52" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V52" s="23"/>
       <c r="Z52" s="23" t="s">
@@ -19888,32 +19888,32 @@
       </c>
       <c r="G53" s="24">
         <f>IF(MIN(Q53,K53,W53)&lt;&gt;0,MIN(Q53,K53,W53),"")</f>
-        <v>0.9847465210875613</v>
+        <v>0.9864585754250055</v>
       </c>
       <c r="H53" s="25">
         <f>IF(AND(ISNUMBER(F53),ISNUMBER(G53)),F53*G53,"")</f>
-        <v>2.9542</v>
+        <v>2.9594</v>
       </c>
       <c r="I53" s="23">
-        <v>8933</v>
+        <v>8867</v>
       </c>
       <c r="J53" s="23"/>
       <c r="K53" s="24">
         <f>IFERROR(IF(OR(J53&gt;=L53,F53&gt;=L53),USD_CHF*LOOKUP(IF(J53="",F53,J53),{0,1,10,25,50,100,250,500,1000,2000},{0.0,0.871,0.669,0.622,0.555,0.482,0.404,0.355,0.308,0.295}),"MOQ="&amp;L53),"")</f>
-        <v>0.9847465210875613</v>
+        <v>0.9864585754250055</v>
       </c>
       <c r="L53" s="23">
         <v>1</v>
       </c>
       <c r="M53" s="25">
         <f>IFERROR(IF(J53="",F53,J53)*K53,"")</f>
-        <v>2.9542</v>
+        <v>2.9594</v>
       </c>
       <c r="N53" s="23" t="s">
         <v>617</v>
       </c>
       <c r="O53" s="23">
-        <v>15095</v>
+        <v>13092</v>
       </c>
       <c r="P53" s="23"/>
       <c r="Q53" s="24">
@@ -19960,25 +19960,25 @@
         <v>0.3</v>
       </c>
       <c r="I54" s="23">
-        <v>1005696</v>
+        <v>985110</v>
       </c>
       <c r="J54" s="23"/>
       <c r="K54" s="24">
         <f>IFERROR(IF(OR(J54&gt;=L54,F54&gt;=L54),USD_CHF*LOOKUP(IF(J54="",F54,J54),{0,1,10,100,1000,2500,10000,50000},{0.0,0.091,0.012,0.007,0.006,0.004,0.004,0.003}),"MOQ="&amp;L54),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L54" s="23">
         <v>1</v>
       </c>
       <c r="M54" s="25">
         <f>IFERROR(IF(J54="",F54,J54)*K54,"")</f>
-        <v>0.3087</v>
+        <v>0.3092</v>
       </c>
       <c r="N54" s="23" t="s">
         <v>618</v>
       </c>
       <c r="O54" s="23">
-        <v>3420298</v>
+        <v>3269541</v>
       </c>
       <c r="P54" s="23"/>
       <c r="Q54" s="24">
@@ -19996,7 +19996,7 @@
         <v>366</v>
       </c>
       <c r="U54" s="23">
-        <v>58370</v>
+        <v>58367</v>
       </c>
       <c r="V54" s="23"/>
       <c r="W54" s="24">
@@ -20036,32 +20036,32 @@
       </c>
       <c r="G55" s="24">
         <f>IF(MIN(Q55,K55,W55)&lt;&gt;0,MIN(Q55,K55,W55),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="H55" s="25">
         <f>IF(AND(ISNUMBER(F55),ISNUMBER(G55)),F55*G55,"")</f>
-        <v>0.1232</v>
+        <v>0.1234</v>
       </c>
       <c r="I55" s="23">
-        <v>461985</v>
+        <v>460545</v>
       </c>
       <c r="J55" s="23"/>
       <c r="K55" s="24">
         <f>IFERROR(IF(OR(J55&gt;=L55,F55&gt;=L55),USD_CHF*LOOKUP(IF(J55="",F55,J55),{0,1,10,100,1000,5000,10000},{0.0,0.109,0.041,0.025,0.02,0.016,0.012}),"MOQ="&amp;L55),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="L55" s="23">
         <v>1</v>
       </c>
       <c r="M55" s="25">
         <f>IFERROR(IF(J55="",F55,J55)*K55,"")</f>
-        <v>0.1232</v>
+        <v>0.1234</v>
       </c>
       <c r="N55" s="23" t="s">
         <v>619</v>
       </c>
       <c r="O55" s="23">
-        <v>1983639</v>
+        <v>1983139</v>
       </c>
       <c r="P55" s="23"/>
       <c r="Q55" s="24">
@@ -20079,11 +20079,11 @@
         <v>374</v>
       </c>
       <c r="U55" s="23">
-        <v>4570</v>
+        <v>4560</v>
       </c>
       <c r="V55" s="23"/>
       <c r="W55" s="24">
-        <f>IFERROR(IF(OR(V55&gt;=X55,F55&gt;=X55),LOOKUP(IF(V55="",F55,V55),{0,1,10,25,50,100,250,500,1000},{0.0,0.0635,0.0635,0.0545,0.0462,0.0379,0.0284,0.0227,0.0212}),"MOQ="&amp;X55),"")</f>
+        <f>IFERROR(IF(OR(V55&gt;=X55,F55&gt;=X55),LOOKUP(IF(V55="",F55,V55),{0,1,10,25,50,100,250,500,1000},{0.0,0.0635,0.0635,0.0546,0.0462,0.0379,0.0284,0.0227,0.0212}),"MOQ="&amp;X55),"")</f>
         <v/>
       </c>
       <c r="X55" s="23">
@@ -20126,19 +20126,19 @@
         <v>1.56</v>
       </c>
       <c r="I56" s="23">
-        <v>7045</v>
+        <v>6935</v>
       </c>
       <c r="J56" s="23"/>
       <c r="K56" s="24">
         <f>IFERROR(IF(OR(J56&gt;=L56,F56&gt;=L56),USD_CHF*LOOKUP(IF(J56="",F56,J56),{0,1,10,100,500,1000,2500,5000,10000,25000},{0.0,0.236,0.107,0.06,0.047,0.032,0.03,0.03,0.025,0.024}),"MOQ="&amp;L56),"")</f>
-        <v>0.2668199529008777</v>
+        <v>0.26728383903593717</v>
       </c>
       <c r="L56" s="23">
         <v>1</v>
       </c>
       <c r="M56" s="25">
         <f>IFERROR(IF(J56="",F56,J56)*K56,"")</f>
-        <v>1.6009</v>
+        <v>1.6037</v>
       </c>
       <c r="N56" s="23" t="s">
         <v>620</v>
@@ -20191,19 +20191,19 @@
         <v>1.2</v>
       </c>
       <c r="I57" s="23">
-        <v>13400</v>
+        <v>13350</v>
       </c>
       <c r="J57" s="23"/>
       <c r="K57" s="24">
         <f>IFERROR(IF(OR(J57&gt;=L57,F57&gt;=L57),USD_CHF*LOOKUP(IF(J57="",F57,J57),{0,1,10,100,1000,5000,10000,25000,50000},{0.0,0.181,0.065,0.04,0.032,0.025,0.024,0.021,0.02}),"MOQ="&amp;L57),"")</f>
-        <v>0.204637336758724</v>
+        <v>0.20499311383688404</v>
       </c>
       <c r="L57" s="23">
         <v>1</v>
       </c>
       <c r="M57" s="25">
         <f>IFERROR(IF(J57="",F57,J57)*K57,"")</f>
-        <v>1.2278</v>
+        <v>1.23</v>
       </c>
       <c r="N57" s="23" t="s">
         <v>621</v>
@@ -20261,14 +20261,14 @@
       <c r="J58" s="23"/>
       <c r="K58" s="24">
         <f>IFERROR(IF(OR(J58&gt;=L58,F58&gt;=L58),USD_CHF*LOOKUP(IF(J58="",F58,J58),{0,1,10,100,1000,5000,10000,50000},{0.0,0.127,0.039,0.025,0.021,0.014,0.013,0.012}),"MOQ="&amp;L58),"")</f>
-        <v>0.14358531363733673</v>
+        <v>0.14383494727781365</v>
       </c>
       <c r="L58" s="23">
         <v>1</v>
       </c>
       <c r="M58" s="25">
         <f>IFERROR(IF(J58="",F58,J58)*K58,"")</f>
-        <v>0.1436</v>
+        <v>0.1438</v>
       </c>
       <c r="N58" s="23" t="s">
         <v>622</v>
@@ -20292,7 +20292,7 @@
         <v>393</v>
       </c>
       <c r="U58" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V58" s="23"/>
       <c r="W58" s="24">
@@ -20339,25 +20339,25 @@
         <v>0.3</v>
       </c>
       <c r="I59" s="23">
-        <v>206603</v>
+        <v>206254</v>
       </c>
       <c r="J59" s="23"/>
       <c r="K59" s="24">
         <f>IFERROR(IF(OR(J59&gt;=L59,F59&gt;=L59),USD_CHF*LOOKUP(IF(J59="",F59,J59),{0,1,10,100,1000,2500,10000,100000},{0.0,0.091,0.014,0.008,0.007,0.006,0.004,0.003}),"MOQ="&amp;L59),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L59" s="23">
         <v>1</v>
       </c>
       <c r="M59" s="25">
         <f>IFERROR(IF(J59="",F59,J59)*K59,"")</f>
-        <v>0.3087</v>
+        <v>0.3092</v>
       </c>
       <c r="N59" s="23" t="s">
         <v>623</v>
       </c>
       <c r="O59" s="23">
-        <v>390221</v>
+        <v>380121</v>
       </c>
       <c r="P59" s="23"/>
       <c r="Q59" s="24">
@@ -20375,7 +20375,7 @@
         <v>399</v>
       </c>
       <c r="U59" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V59" s="23"/>
       <c r="W59" s="24">
@@ -20427,14 +20427,14 @@
       <c r="J60" s="23"/>
       <c r="K60" s="24">
         <f>IFERROR(IF(OR(J60&gt;=L60,F60&gt;=L60),USD_CHF*LOOKUP(IF(J60="",F60,J60),{0,1,10,100,1000,5000,10000,25000},{0.0,0.145,0.047,0.029,0.02,0.017,0.015,0.013}),"MOQ="&amp;L60),"")</f>
-        <v>0.1639359880111325</v>
+        <v>0.16422100279750376</v>
       </c>
       <c r="L60" s="23">
         <v>1</v>
       </c>
       <c r="M60" s="25">
         <f>IFERROR(IF(J60="",F60,J60)*K60,"")</f>
-        <v>0.3279</v>
+        <v>0.3284</v>
       </c>
       <c r="N60" s="23" t="s">
         <v>624</v>
@@ -20480,11 +20480,11 @@
       </c>
       <c r="G61" s="24">
         <f>IF(MIN(Q61,K61,W61)&lt;&gt;0,MIN(Q61,K61,W61),"")</f>
-        <v>0.03504838364375936</v>
+        <v>0.035109317839466324</v>
       </c>
       <c r="H61" s="25">
         <f>IF(AND(ISNUMBER(F61),ISNUMBER(G61)),F61*G61,"")</f>
-        <v>0.4907</v>
+        <v>0.4915</v>
       </c>
       <c r="I61" s="23">
         <v>40368</v>
@@ -20492,14 +20492,14 @@
       <c r="J61" s="23"/>
       <c r="K61" s="24">
         <f>IFERROR(IF(OR(J61&gt;=L61,F61&gt;=L61),USD_CHF*LOOKUP(IF(J61="",F61,J61),{0,1,10,100,1000,2500,10000},{0.0,0.099,0.031,0.019,0.015,0.013,0.012}),"MOQ="&amp;L61),"")</f>
-        <v>0.03504838364375936</v>
+        <v>0.035109317839466324</v>
       </c>
       <c r="L61" s="23">
         <v>1</v>
       </c>
       <c r="M61" s="25">
         <f>IFERROR(IF(J61="",F61,J61)*K61,"")</f>
-        <v>0.4907</v>
+        <v>0.4915</v>
       </c>
       <c r="N61" s="23" t="s">
         <v>625</v>
@@ -20545,32 +20545,32 @@
       </c>
       <c r="G62" s="24">
         <f>IF(MIN(Q62,K62,W62)&lt;&gt;0,MIN(Q62,K62,W62),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="H62" s="25">
         <f>IF(AND(ISNUMBER(F62),ISNUMBER(G62)),F62*G62,"")</f>
-        <v>0.1232</v>
+        <v>0.1234</v>
       </c>
       <c r="I62" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J62" s="23"/>
       <c r="K62" s="24">
         <f>IFERROR(IF(OR(J62&gt;=L62,F62&gt;=L62),USD_CHF*LOOKUP(IF(J62="",F62,J62),{0,1,10,100,2500,10000},{0.0,0.109,0.033,0.02,0.012,0.01}),"MOQ="&amp;L62),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="L62" s="23">
         <v>1</v>
       </c>
       <c r="M62" s="25">
         <f>IFERROR(IF(J62="",F62,J62)*K62,"")</f>
-        <v>0.1232</v>
+        <v>0.1234</v>
       </c>
       <c r="N62" s="23" t="s">
         <v>626</v>
       </c>
       <c r="O62" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="P62" s="23"/>
       <c r="Q62" s="24">
@@ -20617,25 +20617,25 @@
         <v>0.7</v>
       </c>
       <c r="I63" s="23">
-        <v>868580</v>
+        <v>867700</v>
       </c>
       <c r="J63" s="23"/>
       <c r="K63" s="24">
         <f>IFERROR(IF(OR(J63&gt;=L63,F63&gt;=L63),USD_CHF*LOOKUP(IF(J63="",F63,J63),{0,1,10,100,1000,2500,10000},{0.0,0.091,0.015,0.008,0.007,0.006,0.003}),"MOQ="&amp;L63),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L63" s="23">
         <v>1</v>
       </c>
       <c r="M63" s="25">
         <f>IFERROR(IF(J63="",F63,J63)*K63,"")</f>
-        <v>0.7202</v>
+        <v>0.7214</v>
       </c>
       <c r="N63" s="23" t="s">
         <v>627</v>
       </c>
       <c r="O63" s="23">
-        <v>1890935</v>
+        <v>1885578</v>
       </c>
       <c r="P63" s="23"/>
       <c r="Q63" s="24">
@@ -20653,11 +20653,11 @@
         <v>426</v>
       </c>
       <c r="U63" s="23">
-        <v>4770</v>
+        <v>4767</v>
       </c>
       <c r="V63" s="23"/>
       <c r="W63" s="24">
-        <f>IFERROR(IF(OR(V63&gt;=X63,F63&gt;=X63),LOOKUP(IF(V63="",F63,V63),{0,1,8,50,100,1000,2500,10000,500000,1000000},{0.0,0.11,0.0425,0.0152,0.011,0.00524,0.00455,0.00409,0.00384,0.00381}),"MOQ="&amp;X63),"")</f>
+        <f>IFERROR(IF(OR(V63&gt;=X63,F63&gt;=X63),LOOKUP(IF(V63="",F63,V63),{0,1,8,50,100,1000,2500,10000,500000,1000000},{0.0,0.11,0.0425,0.0152,0.011,0.00524,0.00456,0.00409,0.00384,0.00381}),"MOQ="&amp;X63),"")</f>
         <v>0.11</v>
       </c>
       <c r="X63" s="23">
@@ -20705,14 +20705,14 @@
       <c r="J64" s="23"/>
       <c r="K64" s="24">
         <f>IFERROR(IF(OR(J64&gt;=L64,F64&gt;=L64),USD_CHF*LOOKUP(IF(J64="",F64,J64),{0,1,10,100,1000,2500,10000,25000,50000},{0.0,0.091,0.023,0.019,0.013,0.01,0.009,0.007,0.006}),"MOQ="&amp;L64),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L64" s="23">
         <v>1</v>
       </c>
       <c r="M64" s="25">
         <f>IFERROR(IF(J64="",F64,J64)*K64,"")</f>
-        <v>0.1029</v>
+        <v>0.1031</v>
       </c>
       <c r="N64" s="23" t="s">
         <v>628</v>
@@ -20770,14 +20770,14 @@
       <c r="J65" s="23"/>
       <c r="K65" s="24">
         <f>IFERROR(IF(OR(J65&gt;=L65,F65&gt;=L65),USD_CHF*LOOKUP(IF(J65="",F65,J65),{0,1,10,100,1000,2500,10000,20000},{0.0,0.091,0.02,0.015,0.013,0.01,0.007,0.006}),"MOQ="&amp;L65),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L65" s="23">
         <v>1</v>
       </c>
       <c r="M65" s="25">
         <f>IFERROR(IF(J65="",F65,J65)*K65,"")</f>
-        <v>0.1029</v>
+        <v>0.1031</v>
       </c>
       <c r="N65" s="23" t="s">
         <v>629</v>
@@ -20823,32 +20823,32 @@
       </c>
       <c r="G66" s="24">
         <f>IF(MIN(Q66,K66,W66)&lt;&gt;0,MIN(Q66,K66,W66),"")</f>
-        <v>0.0902</v>
+        <v>0.09025</v>
       </c>
       <c r="H66" s="25">
         <f>IF(AND(ISNUMBER(F66),ISNUMBER(G66)),F66*G66,"")</f>
-        <v>0.2706</v>
+        <v>0.2707</v>
       </c>
       <c r="I66" s="23">
-        <v>146709</v>
+        <v>145019</v>
       </c>
       <c r="J66" s="23"/>
       <c r="K66" s="24">
         <f>IFERROR(IF(OR(J66&gt;=L66,F66&gt;=L66),USD_CHF*LOOKUP(IF(J66="",F66,J66),{0,1,10,100,1000,2500,10000},{0.0,0.091,0.02,0.015,0.013,0.01,0.006}),"MOQ="&amp;L66),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L66" s="23">
         <v>1</v>
       </c>
       <c r="M66" s="25">
         <f>IFERROR(IF(J66="",F66,J66)*K66,"")</f>
-        <v>0.3087</v>
+        <v>0.3092</v>
       </c>
       <c r="N66" s="23" t="s">
         <v>630</v>
       </c>
       <c r="O66" s="23">
-        <v>83539</v>
+        <v>83239</v>
       </c>
       <c r="P66" s="23"/>
       <c r="Q66" s="24">
@@ -20870,15 +20870,15 @@
       </c>
       <c r="V66" s="23"/>
       <c r="W66" s="24">
-        <f>IFERROR(IF(OR(V66&gt;=X66,F66&gt;=X66),LOOKUP(IF(V66="",F66,V66),{0,1,10,50,100,500,1000,2500,3000,5000,10000},{0.0,0.0902,0.0211,0.01878,0.01604,0.01466,0.01298,0.01002,0.00971,0.00865,0.0038}),"MOQ="&amp;X66),"")</f>
-        <v>0.0902</v>
+        <f>IFERROR(IF(OR(V66&gt;=X66,F66&gt;=X66),LOOKUP(IF(V66="",F66,V66),{0,1,10,50,100,500,1000,2500,3000,5000,10000},{0.0,0.09025,0.02111,0.01879,0.01604,0.01467,0.01298,0.01003,0.00971,0.00866,0.0038}),"MOQ="&amp;X66),"")</f>
+        <v>0.09025</v>
       </c>
       <c r="X66" s="23">
         <v>1</v>
       </c>
       <c r="Y66" s="25">
         <f>IFERROR(IF(V66="",F66,V66)*W66,"")</f>
-        <v>0.2706</v>
+        <v>0.2707</v>
       </c>
       <c r="Z66" s="23" t="s">
         <v>446</v>
@@ -20913,25 +20913,25 @@
         <v>0.6</v>
       </c>
       <c r="I67" s="23">
-        <v>191994</v>
+        <v>191844</v>
       </c>
       <c r="J67" s="23"/>
       <c r="K67" s="24">
         <f>IFERROR(IF(OR(J67&gt;=L67,F67&gt;=L67),USD_CHF*LOOKUP(IF(J67="",F67,J67),{0,1,10,100,1000,2500,10000,20000},{0.0,0.091,0.02,0.015,0.012,0.009,0.007,0.006}),"MOQ="&amp;L67),"")</f>
-        <v>0.10288396488974522</v>
+        <v>0.1030628362384334</v>
       </c>
       <c r="L67" s="23">
         <v>1</v>
       </c>
       <c r="M67" s="25">
         <f>IFERROR(IF(J67="",F67,J67)*K67,"")</f>
-        <v>0.6173</v>
+        <v>0.6184</v>
       </c>
       <c r="N67" s="23" t="s">
         <v>631</v>
       </c>
       <c r="O67" s="23">
-        <v>74722</v>
+        <v>74472</v>
       </c>
       <c r="P67" s="23"/>
       <c r="Q67" s="24">
@@ -20978,7 +20978,7 @@
         <v>2.66</v>
       </c>
       <c r="I68" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="J68" s="23"/>
       <c r="N68" s="23" t="s">
@@ -21037,14 +21037,14 @@
       <c r="J69" s="23"/>
       <c r="K69" s="24">
         <f>IFERROR(IF(OR(J69&gt;=L69,F69&gt;=L69),USD_CHF*LOOKUP(IF(J69="",F69,J69),{0,1,10,100,500,1000,2500,10000,20000,50000},{0.0,0.109,0.085,0.078,0.067,0.062,0.053,0.047,0.042,0.04}),"MOQ="&amp;L69),"")</f>
-        <v>0.12323463926354097</v>
+        <v>0.12344889175812353</v>
       </c>
       <c r="L69" s="23">
         <v>1</v>
       </c>
       <c r="M69" s="25">
         <f>IFERROR(IF(J69="",F69,J69)*K69,"")</f>
-        <v>0.1232</v>
+        <v>0.1234</v>
       </c>
       <c r="N69" s="23" t="s">
         <v>632</v>
@@ -21072,7 +21072,7 @@
       </c>
       <c r="V69" s="23"/>
       <c r="W69" s="24">
-        <f>IFERROR(IF(OR(V69&gt;=X69,F69&gt;=X69),LOOKUP(IF(V69="",F69,V69),{0,1,10,50,100,500,1000,2500,10000,250000},{0.0,0.13,0.098,0.0808,0.0745,0.0623,0.0581,0.0531,0.0471,0.0377}),"MOQ="&amp;X69),"")</f>
+        <f>IFERROR(IF(OR(V69&gt;=X69,F69&gt;=X69),LOOKUP(IF(V69="",F69,V69),{0,1,10,50,100,500,1000,2500,10000,250000},{0.0,0.13,0.096,0.0798,0.0735,0.0615,0.0573,0.0524,0.0465,0.0372}),"MOQ="&amp;X69),"")</f>
         <v>0.13</v>
       </c>
       <c r="X69" s="23">
@@ -21108,32 +21108,32 @@
       </c>
       <c r="G70" s="24">
         <f>IF(MIN(Q70,K70,W70)&lt;&gt;0,MIN(Q70,K70,W70),"")</f>
-        <v>9.65526439734532</v>
+        <v>9.672050785452981</v>
       </c>
       <c r="H70" s="25">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER(G70)),F70*G70,"")</f>
-        <v>9.6553</v>
+        <v>9.6721</v>
       </c>
       <c r="I70" s="23">
-        <v>6462</v>
+        <v>6446</v>
       </c>
       <c r="J70" s="23"/>
       <c r="K70" s="24">
         <f>IFERROR(IF(OR(J70&gt;=L70,F70&gt;=L70),USD_CHF*LOOKUP(IF(J70="",F70,J70),{0,1,10,100,500,1000},{0.0,8.54,6.31,5.46,4.61,4.51}),"MOQ="&amp;L70),"")</f>
-        <v>9.65526439734532</v>
+        <v>9.672050785452981</v>
       </c>
       <c r="L70" s="23">
         <v>1</v>
       </c>
       <c r="M70" s="25">
         <f>IFERROR(IF(J70="",F70,J70)*K70,"")</f>
-        <v>9.6553</v>
+        <v>9.6721</v>
       </c>
       <c r="N70" s="23" t="s">
         <v>633</v>
       </c>
       <c r="O70" s="23">
-        <v>6428</v>
+        <v>6418</v>
       </c>
       <c r="P70" s="23"/>
       <c r="Q70" s="24">
@@ -21173,11 +21173,11 @@
       </c>
       <c r="G71" s="24">
         <f>IF(MIN(Q71,K71,W71)&lt;&gt;0,MIN(Q71,K71,W71),"")</f>
-        <v>8.242023121387282</v>
+        <v>8.256352485474501</v>
       </c>
       <c r="H71" s="25">
         <f>IF(AND(ISNUMBER(F71),ISNUMBER(G71)),F71*G71,"")</f>
-        <v>8.242</v>
+        <v>8.2564</v>
       </c>
       <c r="I71" s="23">
         <v>2827</v>
@@ -21185,14 +21185,14 @@
       <c r="J71" s="23"/>
       <c r="K71" s="24">
         <f>IFERROR(IF(OR(J71&gt;=L71,F71&gt;=L71),USD_CHF*LOOKUP(IF(J71="",F71,J71),{0,1,10,100,500},{0.0,7.29,5.77,5.32,4.55}),"MOQ="&amp;L71),"")</f>
-        <v>8.242023121387282</v>
+        <v>8.256352485474501</v>
       </c>
       <c r="L71" s="23">
         <v>1</v>
       </c>
       <c r="M71" s="25">
         <f>IFERROR(IF(J71="",F71,J71)*K71,"")</f>
-        <v>8.242</v>
+        <v>8.2564</v>
       </c>
       <c r="N71" s="23" t="s">
         <v>634</v>
@@ -21245,19 +21245,19 @@
         <v>0.93</v>
       </c>
       <c r="I72" s="23">
-        <v>3465</v>
+        <v>3365</v>
       </c>
       <c r="J72" s="23"/>
       <c r="K72" s="24">
         <f>IFERROR(IF(OR(J72&gt;=L72,F72&gt;=L72),USD_CHF*LOOKUP(IF(J72="",F72,J72),{0,1,10,100,500,1000,3000,6000,9000,24000},{0.0,1.08,0.575,0.392,0.356,0.322,0.284,0.265,0.238,0.236}),"MOQ="&amp;L72),"")</f>
-        <v>1.2210404624277456</v>
+        <v>1.2231633311814076</v>
       </c>
       <c r="L72" s="23">
         <v>1</v>
       </c>
       <c r="M72" s="25">
         <f>IFERROR(IF(J72="",F72,J72)*K72,"")</f>
-        <v>1.221</v>
+        <v>1.2232</v>
       </c>
       <c r="N72" s="23" t="s">
         <v>635</v>
@@ -21281,11 +21281,11 @@
         <v>492</v>
       </c>
       <c r="U72" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V72" s="23"/>
       <c r="W72" s="24">
-        <f>IFERROR(IF(OR(V72&gt;=X72,F72&gt;=X72),LOOKUP(IF(V72="",F72,V72),{0,1,5,25,100,500,3000,6000,12000},{0.0,0.93,0.616,0.58,0.547,0.506,0.462,0.43,0.4}),"MOQ="&amp;X72),"")</f>
+        <f>IFERROR(IF(OR(V72&gt;=X72,F72&gt;=X72),LOOKUP(IF(V72="",F72,V72),{0,1,5,25,100,500,3000,6000,12000},{0.0,0.93,0.616,0.58,0.548,0.507,0.462,0.43,0.4}),"MOQ="&amp;X72),"")</f>
         <v>0.93</v>
       </c>
       <c r="X72" s="23">
@@ -21333,14 +21333,14 @@
       <c r="J73" s="23"/>
       <c r="K73" s="24">
         <f>IFERROR(IF(OR(J73&gt;=L73,F73&gt;=L73),USD_CHF*LOOKUP(IF(J73="",F73,J73),{0,1,10,100,250,500,1000,2000,4000},{0.0,5.07,3.58,3.26,3.1,3.0,2.9,2.74,2.71}),"MOQ="&amp;L73),"")</f>
-        <v>5.732106615285805</v>
+        <v>5.7420723047127185</v>
       </c>
       <c r="L73" s="23">
         <v>1</v>
       </c>
       <c r="M73" s="25">
         <f>IFERROR(IF(J73="",F73,J73)*K73,"")</f>
-        <v>5.7321</v>
+        <v>5.7421</v>
       </c>
       <c r="N73" s="23" t="s">
         <v>636</v>
@@ -21398,14 +21398,14 @@
       <c r="J74" s="23"/>
       <c r="K74" s="24">
         <f>IFERROR(IF(OR(J74&gt;=L74,F74&gt;=L74),USD_CHF*LOOKUP(IF(J74="",F74,J74),{0,1,10,100,250,500,1000,2500,5000},{0.0,2.41,1.65,1.48,1.39,1.32,1.28,1.26,1.23}),"MOQ="&amp;L74),"")</f>
-        <v>2.724729180047099</v>
+        <v>2.7294663223585114</v>
       </c>
       <c r="L74" s="23">
         <v>1</v>
       </c>
       <c r="M74" s="25">
         <f>IFERROR(IF(J74="",F74,J74)*K74,"")</f>
-        <v>2.7247</v>
+        <v>2.7295</v>
       </c>
       <c r="N74" s="23" t="s">
         <v>637</v>
@@ -21429,7 +21429,7 @@
         <v>509</v>
       </c>
       <c r="U74" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V74" s="23"/>
       <c r="W74" s="24">
@@ -21481,14 +21481,14 @@
       <c r="J75" s="23"/>
       <c r="K75" s="24">
         <f>IFERROR(IF(OR(J75&gt;=L75,F75&gt;=L75),USD_CHF*LOOKUP(IF(J75="",F75,J75),{0,1,10,100,250,500,1000,3000},{0.0,3.7,2.56,2.32,2.2,2.14,2.08,1.91}),"MOQ="&amp;L75),"")</f>
-        <v>4.183194176835795</v>
+        <v>4.190466967936303</v>
       </c>
       <c r="L75" s="23">
         <v>1</v>
       </c>
       <c r="M75" s="25">
         <f>IFERROR(IF(J75="",F75,J75)*K75,"")</f>
-        <v>4.1832</v>
+        <v>4.1905</v>
       </c>
       <c r="N75" s="23" t="s">
         <v>638</v>
@@ -21512,7 +21512,7 @@
         <v>650</v>
       </c>
       <c r="U75" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V75" s="23"/>
       <c r="W75" s="24">
@@ -21564,14 +21564,14 @@
       <c r="J76" s="23"/>
       <c r="K76" s="24">
         <f>IFERROR(IF(OR(J76&gt;=L76,F76&gt;=L76),USD_CHF*LOOKUP(IF(J76="",F76,J76),{0,1,10,100,500,1000,3000,6000,9000},{0.0,1.25,0.826,0.687,0.661,0.596,0.583,0.575,0.562}),"MOQ="&amp;L76),"")</f>
-        <v>1.4132412759580388</v>
+        <v>1.4156982999784808</v>
       </c>
       <c r="L76" s="23">
         <v>1</v>
       </c>
       <c r="M76" s="25">
         <f>IFERROR(IF(J76="",F76,J76)*K76,"")</f>
-        <v>1.4132</v>
+        <v>1.4157</v>
       </c>
       <c r="N76" s="23" t="s">
         <v>639</v>
@@ -21595,7 +21595,7 @@
         <v>525</v>
       </c>
       <c r="U76" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V76" s="23"/>
       <c r="W76" s="24">
@@ -21642,19 +21642,19 @@
         <v>4.16</v>
       </c>
       <c r="I77" s="23">
-        <v>4812</v>
+        <v>4752</v>
       </c>
       <c r="J77" s="23"/>
       <c r="K77" s="24">
         <f>IFERROR(IF(OR(J77&gt;=L77,F77&gt;=L77),USD_CHF*LOOKUP(IF(J77="",F77,J77),{0,1,10,100,250,500,1000,2500,5000},{0.0,3.77,2.63,2.39,2.26,2.16,2.14,2.06,2.05}),"MOQ="&amp;L77),"")</f>
-        <v>4.262335688289445</v>
+        <v>4.269746072735098</v>
       </c>
       <c r="L77" s="23">
         <v>1</v>
       </c>
       <c r="M77" s="25">
         <f>IFERROR(IF(J77="",F77,J77)*K77,"")</f>
-        <v>4.2623</v>
+        <v>4.2697</v>
       </c>
       <c r="N77" s="23" t="s">
         <v>640</v>
@@ -21678,7 +21678,7 @@
         <v>532</v>
       </c>
       <c r="U77" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V77" s="23"/>
       <c r="Z77" s="23" t="s">
@@ -21719,20 +21719,20 @@
       <c r="J78" s="23"/>
       <c r="K78" s="24">
         <f>IFERROR(IF(OR(J78&gt;=L78,F78&gt;=L78),USD_CHF*LOOKUP(IF(J78="",F78,J78),{0,1,10,25,100,250,500},{0.0,8.12,6.32,5.87,5.17,4.99,4.98}),"MOQ="&amp;L78),"")</f>
-        <v>9.180415328623418</v>
+        <v>9.196376156660211</v>
       </c>
       <c r="L78" s="23">
         <v>1</v>
       </c>
       <c r="M78" s="25">
         <f>IFERROR(IF(J78="",F78,J78)*K78,"")</f>
-        <v>9.1804</v>
+        <v>9.1964</v>
       </c>
       <c r="N78" s="23" t="s">
         <v>641</v>
       </c>
       <c r="O78" s="23">
-        <v>885</v>
+        <v>879</v>
       </c>
       <c r="P78" s="23"/>
       <c r="Q78" s="24">
@@ -21750,19 +21750,19 @@
         <v>540</v>
       </c>
       <c r="U78" s="26" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="V78" s="23"/>
       <c r="W78" s="24">
-        <f>IFERROR(IF(OR(V78&gt;=X78,F78&gt;=X78),LOOKUP(IF(V78="",F78,V78),{0,1,3,10,25,50,100,250,500,1000},{0.0,10.76,10.23,9.73,9.17,8.61,8.05,7.27,6.99,6.71}),"MOQ="&amp;X78),"")</f>
-        <v>10.76</v>
+        <f>IFERROR(IF(OR(V78&gt;=X78,F78&gt;=X78),LOOKUP(IF(V78="",F78,V78),{0,1,3,10,25,50,100,250,500,1000},{0.0,10.77,10.24,9.73,9.17,8.61,8.05,7.27,7,6.71}),"MOQ="&amp;X78),"")</f>
+        <v>10.77</v>
       </c>
       <c r="X78" s="23">
         <v>1</v>
       </c>
       <c r="Y78" s="25">
         <f>IFERROR(IF(V78="",F78,V78)*W78,"")</f>
-        <v>10.76</v>
+        <v>10.77</v>
       </c>
       <c r="Z78" s="23" t="s">
         <v>537</v>
@@ -21802,14 +21802,14 @@
       <c r="J79" s="23"/>
       <c r="K79" s="24">
         <f>IFERROR(IF(OR(J79&gt;=L79,F79&gt;=L79),USD_CHF*LOOKUP(IF(J79="",F79,J79),{0,1,10,100,250,500,1000,3000,6000},{0.0,1.58,1.05,0.943,0.881,0.848,0.821,0.773,0.739}),"MOQ="&amp;L79),"")</f>
-        <v>1.786336972810961</v>
+        <v>1.7894426511727999</v>
       </c>
       <c r="L79" s="23">
         <v>1</v>
       </c>
       <c r="M79" s="25">
         <f>IFERROR(IF(J79="",F79,J79)*K79,"")</f>
-        <v>1.7863</v>
+        <v>1.7894</v>
       </c>
       <c r="N79" s="23" t="s">
         <v>642</v>
@@ -21862,25 +21862,25 @@
         <v>1.17</v>
       </c>
       <c r="I80" s="23">
-        <v>6702</v>
+        <v>6682</v>
       </c>
       <c r="J80" s="23"/>
       <c r="K80" s="24">
         <f>IFERROR(IF(OR(J80&gt;=L80,F80&gt;=L80),USD_CHF*LOOKUP(IF(J80="",F80,J80),{0,1,10,100,500,1000,3000,6000,9000,24000},{0.0,1.06,0.693,0.574,0.551,0.531,0.507,0.487,0.475,0.472}),"MOQ="&amp;L80),"")</f>
-        <v>1.1984286020124169</v>
+        <v>1.200512158381752</v>
       </c>
       <c r="L80" s="23">
         <v>1</v>
       </c>
       <c r="M80" s="25">
         <f>IFERROR(IF(J80="",F80,J80)*K80,"")</f>
-        <v>1.1984</v>
+        <v>1.2005</v>
       </c>
       <c r="N80" s="23" t="s">
         <v>643</v>
       </c>
       <c r="O80" s="23">
-        <v>12393</v>
+        <v>12213</v>
       </c>
       <c r="P80" s="23"/>
       <c r="Q80" s="24">
@@ -21902,7 +21902,7 @@
       </c>
       <c r="V80" s="23"/>
       <c r="W80" s="24">
-        <f>IFERROR(IF(OR(V80&gt;=X80,F80&gt;=X80),LOOKUP(IF(V80="",F80,V80),{0,1,10,50,100,250,500,1000,2500,3000,9000},{0.0,1.225,1.084,0.909,0.832,0.738,0.674,0.615,0.545,0.533,0.523}),"MOQ="&amp;X80),"")</f>
+        <f>IFERROR(IF(OR(V80&gt;=X80,F80&gt;=X80),LOOKUP(IF(V80="",F80,V80),{0,1,10,50,100,250,500,1000,2500,3000,9000},{0.0,1.225,1.085,0.91,0.833,0.739,0.675,0.615,0.546,0.533,0.524}),"MOQ="&amp;X80),"")</f>
         <v>1.225</v>
       </c>
       <c r="X80" s="23">
@@ -21966,7 +21966,7 @@
         <v>661</v>
       </c>
       <c r="C83">
-        <v>1.130593020766431</v>
+        <v>1.132558639982785</v>
       </c>
       <c r="G83" s="27" t="s">
         <v>659</v>

</xml_diff>